<commit_message>
Insert date and plate number in .xlsx sheet before download the file.
</commit_message>
<xml_diff>
--- a/assets/DatabaseTemplate.xlsx
+++ b/assets/DatabaseTemplate.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="220">
   <si>
     <t>1100 รถกะบะบรรทุก</t>
   </si>
@@ -839,7 +839,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -870,7 +869,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -884,18 +883,15 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4007,3166 +4003,638 @@
       <c r="C368" s="1"/>
       <c r="D368" s="1"/>
     </row>
-    <row r="369" ht="15.75" customHeight="1">
-      <c r="B369" s="1"/>
-      <c r="C369" s="1"/>
-      <c r="D369" s="1"/>
-    </row>
-    <row r="370" ht="15.75" customHeight="1">
-      <c r="B370" s="1"/>
-      <c r="C370" s="1"/>
-      <c r="D370" s="1"/>
-    </row>
-    <row r="371" ht="15.75" customHeight="1">
-      <c r="B371" s="1"/>
-      <c r="C371" s="1"/>
-      <c r="D371" s="1"/>
-    </row>
-    <row r="372" ht="15.75" customHeight="1">
-      <c r="B372" s="1"/>
-      <c r="C372" s="1"/>
-      <c r="D372" s="1"/>
-    </row>
-    <row r="373" ht="15.75" customHeight="1">
-      <c r="B373" s="1"/>
-      <c r="C373" s="1"/>
-      <c r="D373" s="1"/>
-    </row>
-    <row r="374" ht="15.75" customHeight="1">
-      <c r="B374" s="1"/>
-      <c r="C374" s="1"/>
-      <c r="D374" s="1"/>
-    </row>
-    <row r="375" ht="15.75" customHeight="1">
-      <c r="B375" s="1"/>
-      <c r="C375" s="1"/>
-      <c r="D375" s="1"/>
-    </row>
-    <row r="376" ht="15.75" customHeight="1">
-      <c r="B376" s="1"/>
-      <c r="C376" s="1"/>
-      <c r="D376" s="1"/>
-    </row>
-    <row r="377" ht="15.75" customHeight="1">
-      <c r="B377" s="1"/>
-      <c r="C377" s="1"/>
-      <c r="D377" s="1"/>
-    </row>
-    <row r="378" ht="15.75" customHeight="1">
-      <c r="B378" s="1"/>
-      <c r="C378" s="1"/>
-      <c r="D378" s="1"/>
-    </row>
-    <row r="379" ht="15.75" customHeight="1">
-      <c r="B379" s="1"/>
-      <c r="C379" s="1"/>
-      <c r="D379" s="1"/>
-    </row>
-    <row r="380" ht="15.75" customHeight="1">
-      <c r="B380" s="1"/>
-      <c r="C380" s="1"/>
-      <c r="D380" s="1"/>
-    </row>
-    <row r="381" ht="15.75" customHeight="1">
-      <c r="B381" s="1"/>
-      <c r="C381" s="1"/>
-      <c r="D381" s="1"/>
-    </row>
-    <row r="382" ht="15.75" customHeight="1">
-      <c r="B382" s="1"/>
-      <c r="C382" s="1"/>
-      <c r="D382" s="1"/>
-    </row>
-    <row r="383" ht="15.75" customHeight="1">
-      <c r="B383" s="1"/>
-      <c r="C383" s="1"/>
-      <c r="D383" s="1"/>
-    </row>
-    <row r="384" ht="15.75" customHeight="1">
-      <c r="B384" s="1"/>
-      <c r="C384" s="1"/>
-      <c r="D384" s="1"/>
-    </row>
-    <row r="385" ht="15.75" customHeight="1">
-      <c r="B385" s="1"/>
-      <c r="C385" s="1"/>
-      <c r="D385" s="1"/>
-    </row>
-    <row r="386" ht="15.75" customHeight="1">
-      <c r="B386" s="1"/>
-      <c r="C386" s="1"/>
-      <c r="D386" s="1"/>
-    </row>
-    <row r="387" ht="15.75" customHeight="1">
-      <c r="B387" s="1"/>
-      <c r="C387" s="1"/>
-      <c r="D387" s="1"/>
-    </row>
-    <row r="388" ht="15.75" customHeight="1">
-      <c r="B388" s="1"/>
-      <c r="C388" s="1"/>
-      <c r="D388" s="1"/>
-    </row>
-    <row r="389" ht="15.75" customHeight="1">
-      <c r="B389" s="1"/>
-      <c r="C389" s="1"/>
-      <c r="D389" s="1"/>
-    </row>
-    <row r="390" ht="15.75" customHeight="1">
-      <c r="B390" s="1"/>
-      <c r="C390" s="1"/>
-      <c r="D390" s="1"/>
-    </row>
-    <row r="391" ht="15.75" customHeight="1">
-      <c r="B391" s="1"/>
-      <c r="C391" s="1"/>
-      <c r="D391" s="1"/>
-    </row>
-    <row r="392" ht="15.75" customHeight="1">
-      <c r="B392" s="1"/>
-      <c r="C392" s="1"/>
-      <c r="D392" s="1"/>
-    </row>
-    <row r="393" ht="15.75" customHeight="1">
-      <c r="B393" s="1"/>
-      <c r="C393" s="1"/>
-      <c r="D393" s="1"/>
-    </row>
-    <row r="394" ht="15.75" customHeight="1">
-      <c r="B394" s="1"/>
-      <c r="C394" s="1"/>
-      <c r="D394" s="1"/>
-    </row>
-    <row r="395" ht="15.75" customHeight="1">
-      <c r="B395" s="1"/>
-      <c r="C395" s="1"/>
-      <c r="D395" s="1"/>
-    </row>
-    <row r="396" ht="15.75" customHeight="1">
-      <c r="B396" s="1"/>
-      <c r="C396" s="1"/>
-      <c r="D396" s="1"/>
-    </row>
-    <row r="397" ht="15.75" customHeight="1">
-      <c r="B397" s="1"/>
-      <c r="C397" s="1"/>
-      <c r="D397" s="1"/>
-    </row>
-    <row r="398" ht="15.75" customHeight="1">
-      <c r="B398" s="1"/>
-      <c r="C398" s="1"/>
-      <c r="D398" s="1"/>
-    </row>
-    <row r="399" ht="15.75" customHeight="1">
-      <c r="B399" s="1"/>
-      <c r="C399" s="1"/>
-      <c r="D399" s="1"/>
-    </row>
-    <row r="400" ht="15.75" customHeight="1">
-      <c r="B400" s="1"/>
-      <c r="C400" s="1"/>
-      <c r="D400" s="1"/>
-    </row>
-    <row r="401" ht="15.75" customHeight="1">
-      <c r="B401" s="1"/>
-      <c r="C401" s="1"/>
-      <c r="D401" s="1"/>
-    </row>
-    <row r="402" ht="15.75" customHeight="1">
-      <c r="B402" s="1"/>
-      <c r="C402" s="1"/>
-      <c r="D402" s="1"/>
-    </row>
-    <row r="403" ht="15.75" customHeight="1">
-      <c r="B403" s="1"/>
-      <c r="C403" s="1"/>
-      <c r="D403" s="1"/>
-    </row>
-    <row r="404" ht="15.75" customHeight="1">
-      <c r="B404" s="1"/>
-      <c r="C404" s="1"/>
-      <c r="D404" s="1"/>
-    </row>
-    <row r="405" ht="15.75" customHeight="1">
-      <c r="B405" s="1"/>
-      <c r="C405" s="1"/>
-      <c r="D405" s="1"/>
-    </row>
-    <row r="406" ht="15.75" customHeight="1">
-      <c r="B406" s="1"/>
-      <c r="C406" s="1"/>
-      <c r="D406" s="1"/>
-    </row>
-    <row r="407" ht="15.75" customHeight="1">
-      <c r="B407" s="1"/>
-      <c r="C407" s="1"/>
-      <c r="D407" s="1"/>
-    </row>
-    <row r="408" ht="15.75" customHeight="1">
-      <c r="B408" s="1"/>
-      <c r="C408" s="1"/>
-      <c r="D408" s="1"/>
-    </row>
-    <row r="409" ht="15.75" customHeight="1">
-      <c r="B409" s="1"/>
-      <c r="C409" s="1"/>
-      <c r="D409" s="1"/>
-    </row>
-    <row r="410" ht="15.75" customHeight="1">
-      <c r="B410" s="1"/>
-      <c r="C410" s="1"/>
-      <c r="D410" s="1"/>
-    </row>
-    <row r="411" ht="15.75" customHeight="1">
-      <c r="B411" s="1"/>
-      <c r="C411" s="1"/>
-      <c r="D411" s="1"/>
-    </row>
-    <row r="412" ht="15.75" customHeight="1">
-      <c r="B412" s="1"/>
-      <c r="C412" s="1"/>
-      <c r="D412" s="1"/>
-    </row>
-    <row r="413" ht="15.75" customHeight="1">
-      <c r="B413" s="1"/>
-      <c r="C413" s="1"/>
-      <c r="D413" s="1"/>
-    </row>
-    <row r="414" ht="15.75" customHeight="1">
-      <c r="B414" s="1"/>
-      <c r="C414" s="1"/>
-      <c r="D414" s="1"/>
-    </row>
-    <row r="415" ht="15.75" customHeight="1">
-      <c r="B415" s="1"/>
-      <c r="C415" s="1"/>
-      <c r="D415" s="1"/>
-    </row>
-    <row r="416" ht="15.75" customHeight="1">
-      <c r="B416" s="1"/>
-      <c r="C416" s="1"/>
-      <c r="D416" s="1"/>
-    </row>
-    <row r="417" ht="15.75" customHeight="1">
-      <c r="B417" s="1"/>
-      <c r="C417" s="1"/>
-      <c r="D417" s="1"/>
-    </row>
-    <row r="418" ht="15.75" customHeight="1">
-      <c r="B418" s="1"/>
-      <c r="C418" s="1"/>
-      <c r="D418" s="1"/>
-    </row>
-    <row r="419" ht="15.75" customHeight="1">
-      <c r="B419" s="1"/>
-      <c r="C419" s="1"/>
-      <c r="D419" s="1"/>
-    </row>
-    <row r="420" ht="15.75" customHeight="1">
-      <c r="B420" s="1"/>
-      <c r="C420" s="1"/>
-      <c r="D420" s="1"/>
-    </row>
-    <row r="421" ht="15.75" customHeight="1">
-      <c r="B421" s="1"/>
-      <c r="C421" s="1"/>
-      <c r="D421" s="1"/>
-    </row>
-    <row r="422" ht="15.75" customHeight="1">
-      <c r="B422" s="1"/>
-      <c r="C422" s="1"/>
-      <c r="D422" s="1"/>
-    </row>
-    <row r="423" ht="15.75" customHeight="1">
-      <c r="B423" s="1"/>
-      <c r="C423" s="1"/>
-      <c r="D423" s="1"/>
-    </row>
-    <row r="424" ht="15.75" customHeight="1">
-      <c r="B424" s="1"/>
-      <c r="C424" s="1"/>
-      <c r="D424" s="1"/>
-    </row>
-    <row r="425" ht="15.75" customHeight="1">
-      <c r="B425" s="1"/>
-      <c r="C425" s="1"/>
-      <c r="D425" s="1"/>
-    </row>
-    <row r="426" ht="15.75" customHeight="1">
-      <c r="B426" s="1"/>
-      <c r="C426" s="1"/>
-      <c r="D426" s="1"/>
-    </row>
-    <row r="427" ht="15.75" customHeight="1">
-      <c r="B427" s="1"/>
-      <c r="C427" s="1"/>
-      <c r="D427" s="1"/>
-    </row>
-    <row r="428" ht="15.75" customHeight="1">
-      <c r="B428" s="1"/>
-      <c r="C428" s="1"/>
-      <c r="D428" s="1"/>
-    </row>
-    <row r="429" ht="15.75" customHeight="1">
-      <c r="B429" s="1"/>
-      <c r="C429" s="1"/>
-      <c r="D429" s="1"/>
-    </row>
-    <row r="430" ht="15.75" customHeight="1">
-      <c r="B430" s="1"/>
-      <c r="C430" s="1"/>
-      <c r="D430" s="1"/>
-    </row>
-    <row r="431" ht="15.75" customHeight="1">
-      <c r="B431" s="1"/>
-      <c r="C431" s="1"/>
-      <c r="D431" s="1"/>
-    </row>
-    <row r="432" ht="15.75" customHeight="1">
-      <c r="B432" s="1"/>
-      <c r="C432" s="1"/>
-      <c r="D432" s="1"/>
-    </row>
-    <row r="433" ht="15.75" customHeight="1">
-      <c r="B433" s="1"/>
-      <c r="C433" s="1"/>
-      <c r="D433" s="1"/>
-    </row>
-    <row r="434" ht="15.75" customHeight="1">
-      <c r="B434" s="1"/>
-      <c r="C434" s="1"/>
-      <c r="D434" s="1"/>
-    </row>
-    <row r="435" ht="15.75" customHeight="1">
-      <c r="B435" s="1"/>
-      <c r="C435" s="1"/>
-      <c r="D435" s="1"/>
-    </row>
-    <row r="436" ht="15.75" customHeight="1">
-      <c r="B436" s="1"/>
-      <c r="C436" s="1"/>
-      <c r="D436" s="1"/>
-    </row>
-    <row r="437" ht="15.75" customHeight="1">
-      <c r="B437" s="1"/>
-      <c r="C437" s="1"/>
-      <c r="D437" s="1"/>
-    </row>
-    <row r="438" ht="15.75" customHeight="1">
-      <c r="B438" s="1"/>
-      <c r="C438" s="1"/>
-      <c r="D438" s="1"/>
-    </row>
-    <row r="439" ht="15.75" customHeight="1">
-      <c r="B439" s="1"/>
-      <c r="C439" s="1"/>
-      <c r="D439" s="1"/>
-    </row>
-    <row r="440" ht="15.75" customHeight="1">
-      <c r="B440" s="1"/>
-      <c r="C440" s="1"/>
-      <c r="D440" s="1"/>
-    </row>
-    <row r="441" ht="15.75" customHeight="1">
-      <c r="B441" s="1"/>
-      <c r="C441" s="1"/>
-      <c r="D441" s="1"/>
-    </row>
-    <row r="442" ht="15.75" customHeight="1">
-      <c r="B442" s="1"/>
-      <c r="C442" s="1"/>
-      <c r="D442" s="1"/>
-    </row>
-    <row r="443" ht="15.75" customHeight="1">
-      <c r="B443" s="1"/>
-      <c r="C443" s="1"/>
-      <c r="D443" s="1"/>
-    </row>
-    <row r="444" ht="15.75" customHeight="1">
-      <c r="B444" s="1"/>
-      <c r="C444" s="1"/>
-      <c r="D444" s="1"/>
-    </row>
-    <row r="445" ht="15.75" customHeight="1">
-      <c r="B445" s="1"/>
-      <c r="C445" s="1"/>
-      <c r="D445" s="1"/>
-    </row>
-    <row r="446" ht="15.75" customHeight="1">
-      <c r="B446" s="1"/>
-      <c r="C446" s="1"/>
-      <c r="D446" s="1"/>
-    </row>
-    <row r="447" ht="15.75" customHeight="1">
-      <c r="B447" s="1"/>
-      <c r="C447" s="1"/>
-      <c r="D447" s="1"/>
-    </row>
-    <row r="448" ht="15.75" customHeight="1">
-      <c r="B448" s="1"/>
-      <c r="C448" s="1"/>
-      <c r="D448" s="1"/>
-    </row>
-    <row r="449" ht="15.75" customHeight="1">
-      <c r="B449" s="1"/>
-      <c r="C449" s="1"/>
-      <c r="D449" s="1"/>
-    </row>
-    <row r="450" ht="15.75" customHeight="1">
-      <c r="B450" s="1"/>
-      <c r="C450" s="1"/>
-      <c r="D450" s="1"/>
-    </row>
-    <row r="451" ht="15.75" customHeight="1">
-      <c r="B451" s="1"/>
-      <c r="C451" s="1"/>
-      <c r="D451" s="1"/>
-    </row>
-    <row r="452" ht="15.75" customHeight="1">
-      <c r="B452" s="1"/>
-      <c r="C452" s="1"/>
-      <c r="D452" s="1"/>
-    </row>
-    <row r="453" ht="15.75" customHeight="1">
-      <c r="B453" s="1"/>
-      <c r="C453" s="1"/>
-      <c r="D453" s="1"/>
-    </row>
-    <row r="454" ht="15.75" customHeight="1">
-      <c r="B454" s="1"/>
-      <c r="C454" s="1"/>
-      <c r="D454" s="1"/>
-    </row>
-    <row r="455" ht="15.75" customHeight="1">
-      <c r="B455" s="1"/>
-      <c r="C455" s="1"/>
-      <c r="D455" s="1"/>
-    </row>
-    <row r="456" ht="15.75" customHeight="1">
-      <c r="B456" s="1"/>
-      <c r="C456" s="1"/>
-      <c r="D456" s="1"/>
-    </row>
-    <row r="457" ht="15.75" customHeight="1">
-      <c r="B457" s="1"/>
-      <c r="C457" s="1"/>
-      <c r="D457" s="1"/>
-    </row>
-    <row r="458" ht="15.75" customHeight="1">
-      <c r="B458" s="1"/>
-      <c r="C458" s="1"/>
-      <c r="D458" s="1"/>
-    </row>
-    <row r="459" ht="15.75" customHeight="1">
-      <c r="B459" s="1"/>
-      <c r="C459" s="1"/>
-      <c r="D459" s="1"/>
-    </row>
-    <row r="460" ht="15.75" customHeight="1">
-      <c r="B460" s="1"/>
-      <c r="C460" s="1"/>
-      <c r="D460" s="1"/>
-    </row>
-    <row r="461" ht="15.75" customHeight="1">
-      <c r="B461" s="1"/>
-      <c r="C461" s="1"/>
-      <c r="D461" s="1"/>
-    </row>
-    <row r="462" ht="15.75" customHeight="1">
-      <c r="B462" s="1"/>
-      <c r="C462" s="1"/>
-      <c r="D462" s="1"/>
-    </row>
-    <row r="463" ht="15.75" customHeight="1">
-      <c r="B463" s="1"/>
-      <c r="C463" s="1"/>
-      <c r="D463" s="1"/>
-    </row>
-    <row r="464" ht="15.75" customHeight="1">
-      <c r="B464" s="1"/>
-      <c r="C464" s="1"/>
-      <c r="D464" s="1"/>
-    </row>
-    <row r="465" ht="15.75" customHeight="1">
-      <c r="B465" s="1"/>
-      <c r="C465" s="1"/>
-      <c r="D465" s="1"/>
-    </row>
-    <row r="466" ht="15.75" customHeight="1">
-      <c r="B466" s="1"/>
-      <c r="C466" s="1"/>
-      <c r="D466" s="1"/>
-    </row>
-    <row r="467" ht="15.75" customHeight="1">
-      <c r="B467" s="1"/>
-      <c r="C467" s="1"/>
-      <c r="D467" s="1"/>
-    </row>
-    <row r="468" ht="15.75" customHeight="1">
-      <c r="B468" s="1"/>
-      <c r="C468" s="1"/>
-      <c r="D468" s="1"/>
-    </row>
-    <row r="469" ht="15.75" customHeight="1">
-      <c r="B469" s="1"/>
-      <c r="C469" s="1"/>
-      <c r="D469" s="1"/>
-    </row>
-    <row r="470" ht="15.75" customHeight="1">
-      <c r="B470" s="1"/>
-      <c r="C470" s="1"/>
-      <c r="D470" s="1"/>
-    </row>
-    <row r="471" ht="15.75" customHeight="1">
-      <c r="B471" s="1"/>
-      <c r="C471" s="1"/>
-      <c r="D471" s="1"/>
-    </row>
-    <row r="472" ht="15.75" customHeight="1">
-      <c r="B472" s="1"/>
-      <c r="C472" s="1"/>
-      <c r="D472" s="1"/>
-    </row>
-    <row r="473" ht="15.75" customHeight="1">
-      <c r="B473" s="1"/>
-      <c r="C473" s="1"/>
-      <c r="D473" s="1"/>
-    </row>
-    <row r="474" ht="15.75" customHeight="1">
-      <c r="B474" s="1"/>
-      <c r="C474" s="1"/>
-      <c r="D474" s="1"/>
-    </row>
-    <row r="475" ht="15.75" customHeight="1">
-      <c r="B475" s="1"/>
-      <c r="C475" s="1"/>
-      <c r="D475" s="1"/>
-    </row>
-    <row r="476" ht="15.75" customHeight="1">
-      <c r="B476" s="1"/>
-      <c r="C476" s="1"/>
-      <c r="D476" s="1"/>
-    </row>
-    <row r="477" ht="15.75" customHeight="1">
-      <c r="B477" s="1"/>
-      <c r="C477" s="1"/>
-      <c r="D477" s="1"/>
-    </row>
-    <row r="478" ht="15.75" customHeight="1">
-      <c r="B478" s="1"/>
-      <c r="C478" s="1"/>
-      <c r="D478" s="1"/>
-    </row>
-    <row r="479" ht="15.75" customHeight="1">
-      <c r="B479" s="1"/>
-      <c r="C479" s="1"/>
-      <c r="D479" s="1"/>
-    </row>
-    <row r="480" ht="15.75" customHeight="1">
-      <c r="B480" s="1"/>
-      <c r="C480" s="1"/>
-      <c r="D480" s="1"/>
-    </row>
-    <row r="481" ht="15.75" customHeight="1">
-      <c r="B481" s="1"/>
-      <c r="C481" s="1"/>
-      <c r="D481" s="1"/>
-    </row>
-    <row r="482" ht="15.75" customHeight="1">
-      <c r="B482" s="1"/>
-      <c r="C482" s="1"/>
-      <c r="D482" s="1"/>
-    </row>
-    <row r="483" ht="15.75" customHeight="1">
-      <c r="B483" s="1"/>
-      <c r="C483" s="1"/>
-      <c r="D483" s="1"/>
-    </row>
-    <row r="484" ht="15.75" customHeight="1">
-      <c r="B484" s="1"/>
-      <c r="C484" s="1"/>
-      <c r="D484" s="1"/>
-    </row>
-    <row r="485" ht="15.75" customHeight="1">
-      <c r="B485" s="1"/>
-      <c r="C485" s="1"/>
-      <c r="D485" s="1"/>
-    </row>
-    <row r="486" ht="15.75" customHeight="1">
-      <c r="B486" s="1"/>
-      <c r="C486" s="1"/>
-      <c r="D486" s="1"/>
-    </row>
-    <row r="487" ht="15.75" customHeight="1">
-      <c r="B487" s="1"/>
-      <c r="C487" s="1"/>
-      <c r="D487" s="1"/>
-    </row>
-    <row r="488" ht="15.75" customHeight="1">
-      <c r="B488" s="1"/>
-      <c r="C488" s="1"/>
-      <c r="D488" s="1"/>
-    </row>
-    <row r="489" ht="15.75" customHeight="1">
-      <c r="B489" s="1"/>
-      <c r="C489" s="1"/>
-      <c r="D489" s="1"/>
-    </row>
-    <row r="490" ht="15.75" customHeight="1">
-      <c r="B490" s="1"/>
-      <c r="C490" s="1"/>
-      <c r="D490" s="1"/>
-    </row>
-    <row r="491" ht="15.75" customHeight="1">
-      <c r="B491" s="1"/>
-      <c r="C491" s="1"/>
-      <c r="D491" s="1"/>
-    </row>
-    <row r="492" ht="15.75" customHeight="1">
-      <c r="B492" s="1"/>
-      <c r="C492" s="1"/>
-      <c r="D492" s="1"/>
-    </row>
-    <row r="493" ht="15.75" customHeight="1">
-      <c r="B493" s="1"/>
-      <c r="C493" s="1"/>
-      <c r="D493" s="1"/>
-    </row>
-    <row r="494" ht="15.75" customHeight="1">
-      <c r="B494" s="1"/>
-      <c r="C494" s="1"/>
-      <c r="D494" s="1"/>
-    </row>
-    <row r="495" ht="15.75" customHeight="1">
-      <c r="B495" s="1"/>
-      <c r="C495" s="1"/>
-      <c r="D495" s="1"/>
-    </row>
-    <row r="496" ht="15.75" customHeight="1">
-      <c r="B496" s="1"/>
-      <c r="C496" s="1"/>
-      <c r="D496" s="1"/>
-    </row>
-    <row r="497" ht="15.75" customHeight="1">
-      <c r="B497" s="1"/>
-      <c r="C497" s="1"/>
-      <c r="D497" s="1"/>
-    </row>
-    <row r="498" ht="15.75" customHeight="1">
-      <c r="B498" s="1"/>
-      <c r="C498" s="1"/>
-      <c r="D498" s="1"/>
-    </row>
-    <row r="499" ht="15.75" customHeight="1">
-      <c r="B499" s="1"/>
-      <c r="C499" s="1"/>
-      <c r="D499" s="1"/>
-    </row>
-    <row r="500" ht="15.75" customHeight="1">
-      <c r="B500" s="1"/>
-      <c r="C500" s="1"/>
-      <c r="D500" s="1"/>
-    </row>
-    <row r="501" ht="15.75" customHeight="1">
-      <c r="B501" s="1"/>
-      <c r="C501" s="1"/>
-      <c r="D501" s="1"/>
-    </row>
-    <row r="502" ht="15.75" customHeight="1">
-      <c r="B502" s="1"/>
-      <c r="C502" s="1"/>
-      <c r="D502" s="1"/>
-    </row>
-    <row r="503" ht="15.75" customHeight="1">
-      <c r="B503" s="1"/>
-      <c r="C503" s="1"/>
-      <c r="D503" s="1"/>
-    </row>
-    <row r="504" ht="15.75" customHeight="1">
-      <c r="B504" s="1"/>
-      <c r="C504" s="1"/>
-      <c r="D504" s="1"/>
-    </row>
-    <row r="505" ht="15.75" customHeight="1">
-      <c r="B505" s="1"/>
-      <c r="C505" s="1"/>
-      <c r="D505" s="1"/>
-    </row>
-    <row r="506" ht="15.75" customHeight="1">
-      <c r="B506" s="1"/>
-      <c r="C506" s="1"/>
-      <c r="D506" s="1"/>
-    </row>
-    <row r="507" ht="15.75" customHeight="1">
-      <c r="B507" s="1"/>
-      <c r="C507" s="1"/>
-      <c r="D507" s="1"/>
-    </row>
-    <row r="508" ht="15.75" customHeight="1">
-      <c r="B508" s="1"/>
-      <c r="C508" s="1"/>
-      <c r="D508" s="1"/>
-    </row>
-    <row r="509" ht="15.75" customHeight="1">
-      <c r="B509" s="1"/>
-      <c r="C509" s="1"/>
-      <c r="D509" s="1"/>
-    </row>
-    <row r="510" ht="15.75" customHeight="1">
-      <c r="B510" s="1"/>
-      <c r="C510" s="1"/>
-      <c r="D510" s="1"/>
-    </row>
-    <row r="511" ht="15.75" customHeight="1">
-      <c r="B511" s="1"/>
-      <c r="C511" s="1"/>
-      <c r="D511" s="1"/>
-    </row>
-    <row r="512" ht="15.75" customHeight="1">
-      <c r="B512" s="1"/>
-      <c r="C512" s="1"/>
-      <c r="D512" s="1"/>
-    </row>
-    <row r="513" ht="15.75" customHeight="1">
-      <c r="B513" s="1"/>
-      <c r="C513" s="1"/>
-      <c r="D513" s="1"/>
-    </row>
-    <row r="514" ht="15.75" customHeight="1">
-      <c r="B514" s="1"/>
-      <c r="C514" s="1"/>
-      <c r="D514" s="1"/>
-    </row>
-    <row r="515" ht="15.75" customHeight="1">
-      <c r="B515" s="1"/>
-      <c r="C515" s="1"/>
-      <c r="D515" s="1"/>
-    </row>
-    <row r="516" ht="15.75" customHeight="1">
-      <c r="B516" s="1"/>
-      <c r="C516" s="1"/>
-      <c r="D516" s="1"/>
-    </row>
-    <row r="517" ht="15.75" customHeight="1">
-      <c r="B517" s="1"/>
-      <c r="C517" s="1"/>
-      <c r="D517" s="1"/>
-    </row>
-    <row r="518" ht="15.75" customHeight="1">
-      <c r="B518" s="1"/>
-      <c r="C518" s="1"/>
-      <c r="D518" s="1"/>
-    </row>
-    <row r="519" ht="15.75" customHeight="1">
-      <c r="B519" s="1"/>
-      <c r="C519" s="1"/>
-      <c r="D519" s="1"/>
-    </row>
-    <row r="520" ht="15.75" customHeight="1">
-      <c r="B520" s="1"/>
-      <c r="C520" s="1"/>
-      <c r="D520" s="1"/>
-    </row>
-    <row r="521" ht="15.75" customHeight="1">
-      <c r="B521" s="1"/>
-      <c r="C521" s="1"/>
-      <c r="D521" s="1"/>
-    </row>
-    <row r="522" ht="15.75" customHeight="1">
-      <c r="B522" s="1"/>
-      <c r="C522" s="1"/>
-      <c r="D522" s="1"/>
-    </row>
-    <row r="523" ht="15.75" customHeight="1">
-      <c r="B523" s="1"/>
-      <c r="C523" s="1"/>
-      <c r="D523" s="1"/>
-    </row>
-    <row r="524" ht="15.75" customHeight="1">
-      <c r="B524" s="1"/>
-      <c r="C524" s="1"/>
-      <c r="D524" s="1"/>
-    </row>
-    <row r="525" ht="15.75" customHeight="1">
-      <c r="B525" s="1"/>
-      <c r="C525" s="1"/>
-      <c r="D525" s="1"/>
-    </row>
-    <row r="526" ht="15.75" customHeight="1">
-      <c r="B526" s="1"/>
-      <c r="C526" s="1"/>
-      <c r="D526" s="1"/>
-    </row>
-    <row r="527" ht="15.75" customHeight="1">
-      <c r="B527" s="1"/>
-      <c r="C527" s="1"/>
-      <c r="D527" s="1"/>
-    </row>
-    <row r="528" ht="15.75" customHeight="1">
-      <c r="B528" s="1"/>
-      <c r="C528" s="1"/>
-      <c r="D528" s="1"/>
-    </row>
-    <row r="529" ht="15.75" customHeight="1">
-      <c r="B529" s="1"/>
-      <c r="C529" s="1"/>
-      <c r="D529" s="1"/>
-    </row>
-    <row r="530" ht="15.75" customHeight="1">
-      <c r="B530" s="1"/>
-      <c r="C530" s="1"/>
-      <c r="D530" s="1"/>
-    </row>
-    <row r="531" ht="15.75" customHeight="1">
-      <c r="B531" s="1"/>
-      <c r="C531" s="1"/>
-      <c r="D531" s="1"/>
-    </row>
-    <row r="532" ht="15.75" customHeight="1">
-      <c r="B532" s="1"/>
-      <c r="C532" s="1"/>
-      <c r="D532" s="1"/>
-    </row>
-    <row r="533" ht="15.75" customHeight="1">
-      <c r="B533" s="1"/>
-      <c r="C533" s="1"/>
-      <c r="D533" s="1"/>
-    </row>
-    <row r="534" ht="15.75" customHeight="1">
-      <c r="B534" s="1"/>
-      <c r="C534" s="1"/>
-      <c r="D534" s="1"/>
-    </row>
-    <row r="535" ht="15.75" customHeight="1">
-      <c r="B535" s="1"/>
-      <c r="C535" s="1"/>
-      <c r="D535" s="1"/>
-    </row>
-    <row r="536" ht="15.75" customHeight="1">
-      <c r="B536" s="1"/>
-      <c r="C536" s="1"/>
-      <c r="D536" s="1"/>
-    </row>
-    <row r="537" ht="15.75" customHeight="1">
-      <c r="B537" s="1"/>
-      <c r="C537" s="1"/>
-      <c r="D537" s="1"/>
-    </row>
-    <row r="538" ht="15.75" customHeight="1">
-      <c r="B538" s="1"/>
-      <c r="C538" s="1"/>
-      <c r="D538" s="1"/>
-    </row>
-    <row r="539" ht="15.75" customHeight="1">
-      <c r="B539" s="1"/>
-      <c r="C539" s="1"/>
-      <c r="D539" s="1"/>
-    </row>
-    <row r="540" ht="15.75" customHeight="1">
-      <c r="B540" s="1"/>
-      <c r="C540" s="1"/>
-      <c r="D540" s="1"/>
-    </row>
-    <row r="541" ht="15.75" customHeight="1">
-      <c r="B541" s="1"/>
-      <c r="C541" s="1"/>
-      <c r="D541" s="1"/>
-    </row>
-    <row r="542" ht="15.75" customHeight="1">
-      <c r="B542" s="1"/>
-      <c r="C542" s="1"/>
-      <c r="D542" s="1"/>
-    </row>
-    <row r="543" ht="15.75" customHeight="1">
-      <c r="B543" s="1"/>
-      <c r="C543" s="1"/>
-      <c r="D543" s="1"/>
-    </row>
-    <row r="544" ht="15.75" customHeight="1">
-      <c r="B544" s="1"/>
-      <c r="C544" s="1"/>
-      <c r="D544" s="1"/>
-    </row>
-    <row r="545" ht="15.75" customHeight="1">
-      <c r="B545" s="1"/>
-      <c r="C545" s="1"/>
-      <c r="D545" s="1"/>
-    </row>
-    <row r="546" ht="15.75" customHeight="1">
-      <c r="B546" s="1"/>
-      <c r="C546" s="1"/>
-      <c r="D546" s="1"/>
-    </row>
-    <row r="547" ht="15.75" customHeight="1">
-      <c r="B547" s="1"/>
-      <c r="C547" s="1"/>
-      <c r="D547" s="1"/>
-    </row>
-    <row r="548" ht="15.75" customHeight="1">
-      <c r="B548" s="1"/>
-      <c r="C548" s="1"/>
-      <c r="D548" s="1"/>
-    </row>
-    <row r="549" ht="15.75" customHeight="1">
-      <c r="B549" s="1"/>
-      <c r="C549" s="1"/>
-      <c r="D549" s="1"/>
-    </row>
-    <row r="550" ht="15.75" customHeight="1">
-      <c r="B550" s="1"/>
-      <c r="C550" s="1"/>
-      <c r="D550" s="1"/>
-    </row>
-    <row r="551" ht="15.75" customHeight="1">
-      <c r="B551" s="1"/>
-      <c r="C551" s="1"/>
-      <c r="D551" s="1"/>
-    </row>
-    <row r="552" ht="15.75" customHeight="1">
-      <c r="B552" s="1"/>
-      <c r="C552" s="1"/>
-      <c r="D552" s="1"/>
-    </row>
-    <row r="553" ht="15.75" customHeight="1">
-      <c r="B553" s="1"/>
-      <c r="C553" s="1"/>
-      <c r="D553" s="1"/>
-    </row>
-    <row r="554" ht="15.75" customHeight="1">
-      <c r="B554" s="1"/>
-      <c r="C554" s="1"/>
-      <c r="D554" s="1"/>
-    </row>
-    <row r="555" ht="15.75" customHeight="1">
-      <c r="B555" s="1"/>
-      <c r="C555" s="1"/>
-      <c r="D555" s="1"/>
-    </row>
-    <row r="556" ht="15.75" customHeight="1">
-      <c r="B556" s="1"/>
-      <c r="C556" s="1"/>
-      <c r="D556" s="1"/>
-    </row>
-    <row r="557" ht="15.75" customHeight="1">
-      <c r="B557" s="1"/>
-      <c r="C557" s="1"/>
-      <c r="D557" s="1"/>
-    </row>
-    <row r="558" ht="15.75" customHeight="1">
-      <c r="B558" s="1"/>
-      <c r="C558" s="1"/>
-      <c r="D558" s="1"/>
-    </row>
-    <row r="559" ht="15.75" customHeight="1">
-      <c r="B559" s="1"/>
-      <c r="C559" s="1"/>
-      <c r="D559" s="1"/>
-    </row>
-    <row r="560" ht="15.75" customHeight="1">
-      <c r="B560" s="1"/>
-      <c r="C560" s="1"/>
-      <c r="D560" s="1"/>
-    </row>
-    <row r="561" ht="15.75" customHeight="1">
-      <c r="B561" s="1"/>
-      <c r="C561" s="1"/>
-      <c r="D561" s="1"/>
-    </row>
-    <row r="562" ht="15.75" customHeight="1">
-      <c r="B562" s="1"/>
-      <c r="C562" s="1"/>
-      <c r="D562" s="1"/>
-    </row>
-    <row r="563" ht="15.75" customHeight="1">
-      <c r="B563" s="1"/>
-      <c r="C563" s="1"/>
-      <c r="D563" s="1"/>
-    </row>
-    <row r="564" ht="15.75" customHeight="1">
-      <c r="B564" s="1"/>
-      <c r="C564" s="1"/>
-      <c r="D564" s="1"/>
-    </row>
-    <row r="565" ht="15.75" customHeight="1">
-      <c r="B565" s="1"/>
-      <c r="C565" s="1"/>
-      <c r="D565" s="1"/>
-    </row>
-    <row r="566" ht="15.75" customHeight="1">
-      <c r="B566" s="1"/>
-      <c r="C566" s="1"/>
-      <c r="D566" s="1"/>
-    </row>
-    <row r="567" ht="15.75" customHeight="1">
-      <c r="B567" s="1"/>
-      <c r="C567" s="1"/>
-      <c r="D567" s="1"/>
-    </row>
-    <row r="568" ht="15.75" customHeight="1">
-      <c r="B568" s="1"/>
-      <c r="C568" s="1"/>
-      <c r="D568" s="1"/>
-    </row>
-    <row r="569" ht="15.75" customHeight="1">
-      <c r="B569" s="1"/>
-      <c r="C569" s="1"/>
-      <c r="D569" s="1"/>
-    </row>
-    <row r="570" ht="15.75" customHeight="1">
-      <c r="B570" s="1"/>
-      <c r="C570" s="1"/>
-      <c r="D570" s="1"/>
-    </row>
-    <row r="571" ht="15.75" customHeight="1">
-      <c r="B571" s="1"/>
-      <c r="C571" s="1"/>
-      <c r="D571" s="1"/>
-    </row>
-    <row r="572" ht="15.75" customHeight="1">
-      <c r="B572" s="1"/>
-      <c r="C572" s="1"/>
-      <c r="D572" s="1"/>
-    </row>
-    <row r="573" ht="15.75" customHeight="1">
-      <c r="B573" s="1"/>
-      <c r="C573" s="1"/>
-      <c r="D573" s="1"/>
-    </row>
-    <row r="574" ht="15.75" customHeight="1">
-      <c r="B574" s="1"/>
-      <c r="C574" s="1"/>
-      <c r="D574" s="1"/>
-    </row>
-    <row r="575" ht="15.75" customHeight="1">
-      <c r="B575" s="1"/>
-      <c r="C575" s="1"/>
-      <c r="D575" s="1"/>
-    </row>
-    <row r="576" ht="15.75" customHeight="1">
-      <c r="B576" s="1"/>
-      <c r="C576" s="1"/>
-      <c r="D576" s="1"/>
-    </row>
-    <row r="577" ht="15.75" customHeight="1">
-      <c r="B577" s="1"/>
-      <c r="C577" s="1"/>
-      <c r="D577" s="1"/>
-    </row>
-    <row r="578" ht="15.75" customHeight="1">
-      <c r="B578" s="1"/>
-      <c r="C578" s="1"/>
-      <c r="D578" s="1"/>
-    </row>
-    <row r="579" ht="15.75" customHeight="1">
-      <c r="B579" s="1"/>
-      <c r="C579" s="1"/>
-      <c r="D579" s="1"/>
-    </row>
-    <row r="580" ht="15.75" customHeight="1">
-      <c r="B580" s="1"/>
-      <c r="C580" s="1"/>
-      <c r="D580" s="1"/>
-    </row>
-    <row r="581" ht="15.75" customHeight="1">
-      <c r="B581" s="1"/>
-      <c r="C581" s="1"/>
-      <c r="D581" s="1"/>
-    </row>
-    <row r="582" ht="15.75" customHeight="1">
-      <c r="B582" s="1"/>
-      <c r="C582" s="1"/>
-      <c r="D582" s="1"/>
-    </row>
-    <row r="583" ht="15.75" customHeight="1">
-      <c r="B583" s="1"/>
-      <c r="C583" s="1"/>
-      <c r="D583" s="1"/>
-    </row>
-    <row r="584" ht="15.75" customHeight="1">
-      <c r="B584" s="1"/>
-      <c r="C584" s="1"/>
-      <c r="D584" s="1"/>
-    </row>
-    <row r="585" ht="15.75" customHeight="1">
-      <c r="B585" s="1"/>
-      <c r="C585" s="1"/>
-      <c r="D585" s="1"/>
-    </row>
-    <row r="586" ht="15.75" customHeight="1">
-      <c r="B586" s="1"/>
-      <c r="C586" s="1"/>
-      <c r="D586" s="1"/>
-    </row>
-    <row r="587" ht="15.75" customHeight="1">
-      <c r="B587" s="1"/>
-      <c r="C587" s="1"/>
-      <c r="D587" s="1"/>
-    </row>
-    <row r="588" ht="15.75" customHeight="1">
-      <c r="B588" s="1"/>
-      <c r="C588" s="1"/>
-      <c r="D588" s="1"/>
-    </row>
-    <row r="589" ht="15.75" customHeight="1">
-      <c r="B589" s="1"/>
-      <c r="C589" s="1"/>
-      <c r="D589" s="1"/>
-    </row>
-    <row r="590" ht="15.75" customHeight="1">
-      <c r="B590" s="1"/>
-      <c r="C590" s="1"/>
-      <c r="D590" s="1"/>
-    </row>
-    <row r="591" ht="15.75" customHeight="1">
-      <c r="B591" s="1"/>
-      <c r="C591" s="1"/>
-      <c r="D591" s="1"/>
-    </row>
-    <row r="592" ht="15.75" customHeight="1">
-      <c r="B592" s="1"/>
-      <c r="C592" s="1"/>
-      <c r="D592" s="1"/>
-    </row>
-    <row r="593" ht="15.75" customHeight="1">
-      <c r="B593" s="1"/>
-      <c r="C593" s="1"/>
-      <c r="D593" s="1"/>
-    </row>
-    <row r="594" ht="15.75" customHeight="1">
-      <c r="B594" s="1"/>
-      <c r="C594" s="1"/>
-      <c r="D594" s="1"/>
-    </row>
-    <row r="595" ht="15.75" customHeight="1">
-      <c r="B595" s="1"/>
-      <c r="C595" s="1"/>
-      <c r="D595" s="1"/>
-    </row>
-    <row r="596" ht="15.75" customHeight="1">
-      <c r="B596" s="1"/>
-      <c r="C596" s="1"/>
-      <c r="D596" s="1"/>
-    </row>
-    <row r="597" ht="15.75" customHeight="1">
-      <c r="B597" s="1"/>
-      <c r="C597" s="1"/>
-      <c r="D597" s="1"/>
-    </row>
-    <row r="598" ht="15.75" customHeight="1">
-      <c r="B598" s="1"/>
-      <c r="C598" s="1"/>
-      <c r="D598" s="1"/>
-    </row>
-    <row r="599" ht="15.75" customHeight="1">
-      <c r="B599" s="1"/>
-      <c r="C599" s="1"/>
-      <c r="D599" s="1"/>
-    </row>
-    <row r="600" ht="15.75" customHeight="1">
-      <c r="B600" s="1"/>
-      <c r="C600" s="1"/>
-      <c r="D600" s="1"/>
-    </row>
-    <row r="601" ht="15.75" customHeight="1">
-      <c r="B601" s="1"/>
-      <c r="C601" s="1"/>
-      <c r="D601" s="1"/>
-    </row>
-    <row r="602" ht="15.75" customHeight="1">
-      <c r="B602" s="1"/>
-      <c r="C602" s="1"/>
-      <c r="D602" s="1"/>
-    </row>
-    <row r="603" ht="15.75" customHeight="1">
-      <c r="B603" s="1"/>
-      <c r="C603" s="1"/>
-      <c r="D603" s="1"/>
-    </row>
-    <row r="604" ht="15.75" customHeight="1">
-      <c r="B604" s="1"/>
-      <c r="C604" s="1"/>
-      <c r="D604" s="1"/>
-    </row>
-    <row r="605" ht="15.75" customHeight="1">
-      <c r="B605" s="1"/>
-      <c r="C605" s="1"/>
-      <c r="D605" s="1"/>
-    </row>
-    <row r="606" ht="15.75" customHeight="1">
-      <c r="B606" s="1"/>
-      <c r="C606" s="1"/>
-      <c r="D606" s="1"/>
-    </row>
-    <row r="607" ht="15.75" customHeight="1">
-      <c r="B607" s="1"/>
-      <c r="C607" s="1"/>
-      <c r="D607" s="1"/>
-    </row>
-    <row r="608" ht="15.75" customHeight="1">
-      <c r="B608" s="1"/>
-      <c r="C608" s="1"/>
-      <c r="D608" s="1"/>
-    </row>
-    <row r="609" ht="15.75" customHeight="1">
-      <c r="B609" s="1"/>
-      <c r="C609" s="1"/>
-      <c r="D609" s="1"/>
-    </row>
-    <row r="610" ht="15.75" customHeight="1">
-      <c r="B610" s="1"/>
-      <c r="C610" s="1"/>
-      <c r="D610" s="1"/>
-    </row>
-    <row r="611" ht="15.75" customHeight="1">
-      <c r="B611" s="1"/>
-      <c r="C611" s="1"/>
-      <c r="D611" s="1"/>
-    </row>
-    <row r="612" ht="15.75" customHeight="1">
-      <c r="B612" s="1"/>
-      <c r="C612" s="1"/>
-      <c r="D612" s="1"/>
-    </row>
-    <row r="613" ht="15.75" customHeight="1">
-      <c r="B613" s="1"/>
-      <c r="C613" s="1"/>
-      <c r="D613" s="1"/>
-    </row>
-    <row r="614" ht="15.75" customHeight="1">
-      <c r="B614" s="1"/>
-      <c r="C614" s="1"/>
-      <c r="D614" s="1"/>
-    </row>
-    <row r="615" ht="15.75" customHeight="1">
-      <c r="B615" s="1"/>
-      <c r="C615" s="1"/>
-      <c r="D615" s="1"/>
-    </row>
-    <row r="616" ht="15.75" customHeight="1">
-      <c r="B616" s="1"/>
-      <c r="C616" s="1"/>
-      <c r="D616" s="1"/>
-    </row>
-    <row r="617" ht="15.75" customHeight="1">
-      <c r="B617" s="1"/>
-      <c r="C617" s="1"/>
-      <c r="D617" s="1"/>
-    </row>
-    <row r="618" ht="15.75" customHeight="1">
-      <c r="B618" s="1"/>
-      <c r="C618" s="1"/>
-      <c r="D618" s="1"/>
-    </row>
-    <row r="619" ht="15.75" customHeight="1">
-      <c r="B619" s="1"/>
-      <c r="C619" s="1"/>
-      <c r="D619" s="1"/>
-    </row>
-    <row r="620" ht="15.75" customHeight="1">
-      <c r="B620" s="1"/>
-      <c r="C620" s="1"/>
-      <c r="D620" s="1"/>
-    </row>
-    <row r="621" ht="15.75" customHeight="1">
-      <c r="B621" s="1"/>
-      <c r="C621" s="1"/>
-      <c r="D621" s="1"/>
-    </row>
-    <row r="622" ht="15.75" customHeight="1">
-      <c r="B622" s="1"/>
-      <c r="C622" s="1"/>
-      <c r="D622" s="1"/>
-    </row>
-    <row r="623" ht="15.75" customHeight="1">
-      <c r="B623" s="1"/>
-      <c r="C623" s="1"/>
-      <c r="D623" s="1"/>
-    </row>
-    <row r="624" ht="15.75" customHeight="1">
-      <c r="B624" s="1"/>
-      <c r="C624" s="1"/>
-      <c r="D624" s="1"/>
-    </row>
-    <row r="625" ht="15.75" customHeight="1">
-      <c r="B625" s="1"/>
-      <c r="C625" s="1"/>
-      <c r="D625" s="1"/>
-    </row>
-    <row r="626" ht="15.75" customHeight="1">
-      <c r="B626" s="1"/>
-      <c r="C626" s="1"/>
-      <c r="D626" s="1"/>
-    </row>
-    <row r="627" ht="15.75" customHeight="1">
-      <c r="B627" s="1"/>
-      <c r="C627" s="1"/>
-      <c r="D627" s="1"/>
-    </row>
-    <row r="628" ht="15.75" customHeight="1">
-      <c r="B628" s="1"/>
-      <c r="C628" s="1"/>
-      <c r="D628" s="1"/>
-    </row>
-    <row r="629" ht="15.75" customHeight="1">
-      <c r="B629" s="1"/>
-      <c r="C629" s="1"/>
-      <c r="D629" s="1"/>
-    </row>
-    <row r="630" ht="15.75" customHeight="1">
-      <c r="B630" s="1"/>
-      <c r="C630" s="1"/>
-      <c r="D630" s="1"/>
-    </row>
-    <row r="631" ht="15.75" customHeight="1">
-      <c r="B631" s="1"/>
-      <c r="C631" s="1"/>
-      <c r="D631" s="1"/>
-    </row>
-    <row r="632" ht="15.75" customHeight="1">
-      <c r="B632" s="1"/>
-      <c r="C632" s="1"/>
-      <c r="D632" s="1"/>
-    </row>
-    <row r="633" ht="15.75" customHeight="1">
-      <c r="B633" s="1"/>
-      <c r="C633" s="1"/>
-      <c r="D633" s="1"/>
-    </row>
-    <row r="634" ht="15.75" customHeight="1">
-      <c r="B634" s="1"/>
-      <c r="C634" s="1"/>
-      <c r="D634" s="1"/>
-    </row>
-    <row r="635" ht="15.75" customHeight="1">
-      <c r="B635" s="1"/>
-      <c r="C635" s="1"/>
-      <c r="D635" s="1"/>
-    </row>
-    <row r="636" ht="15.75" customHeight="1">
-      <c r="B636" s="1"/>
-      <c r="C636" s="1"/>
-      <c r="D636" s="1"/>
-    </row>
-    <row r="637" ht="15.75" customHeight="1">
-      <c r="B637" s="1"/>
-      <c r="C637" s="1"/>
-      <c r="D637" s="1"/>
-    </row>
-    <row r="638" ht="15.75" customHeight="1">
-      <c r="B638" s="1"/>
-      <c r="C638" s="1"/>
-      <c r="D638" s="1"/>
-    </row>
-    <row r="639" ht="15.75" customHeight="1">
-      <c r="B639" s="1"/>
-      <c r="C639" s="1"/>
-      <c r="D639" s="1"/>
-    </row>
-    <row r="640" ht="15.75" customHeight="1">
-      <c r="B640" s="1"/>
-      <c r="C640" s="1"/>
-      <c r="D640" s="1"/>
-    </row>
-    <row r="641" ht="15.75" customHeight="1">
-      <c r="B641" s="1"/>
-      <c r="C641" s="1"/>
-      <c r="D641" s="1"/>
-    </row>
-    <row r="642" ht="15.75" customHeight="1">
-      <c r="B642" s="1"/>
-      <c r="C642" s="1"/>
-      <c r="D642" s="1"/>
-    </row>
-    <row r="643" ht="15.75" customHeight="1">
-      <c r="B643" s="1"/>
-      <c r="C643" s="1"/>
-      <c r="D643" s="1"/>
-    </row>
-    <row r="644" ht="15.75" customHeight="1">
-      <c r="B644" s="1"/>
-      <c r="C644" s="1"/>
-      <c r="D644" s="1"/>
-    </row>
-    <row r="645" ht="15.75" customHeight="1">
-      <c r="B645" s="1"/>
-      <c r="C645" s="1"/>
-      <c r="D645" s="1"/>
-    </row>
-    <row r="646" ht="15.75" customHeight="1">
-      <c r="B646" s="1"/>
-      <c r="C646" s="1"/>
-      <c r="D646" s="1"/>
-    </row>
-    <row r="647" ht="15.75" customHeight="1">
-      <c r="B647" s="1"/>
-      <c r="C647" s="1"/>
-      <c r="D647" s="1"/>
-    </row>
-    <row r="648" ht="15.75" customHeight="1">
-      <c r="B648" s="1"/>
-      <c r="C648" s="1"/>
-      <c r="D648" s="1"/>
-    </row>
-    <row r="649" ht="15.75" customHeight="1">
-      <c r="B649" s="1"/>
-      <c r="C649" s="1"/>
-      <c r="D649" s="1"/>
-    </row>
-    <row r="650" ht="15.75" customHeight="1">
-      <c r="B650" s="1"/>
-      <c r="C650" s="1"/>
-      <c r="D650" s="1"/>
-    </row>
-    <row r="651" ht="15.75" customHeight="1">
-      <c r="B651" s="1"/>
-      <c r="C651" s="1"/>
-      <c r="D651" s="1"/>
-    </row>
-    <row r="652" ht="15.75" customHeight="1">
-      <c r="B652" s="1"/>
-      <c r="C652" s="1"/>
-      <c r="D652" s="1"/>
-    </row>
-    <row r="653" ht="15.75" customHeight="1">
-      <c r="B653" s="1"/>
-      <c r="C653" s="1"/>
-      <c r="D653" s="1"/>
-    </row>
-    <row r="654" ht="15.75" customHeight="1">
-      <c r="B654" s="1"/>
-      <c r="C654" s="1"/>
-      <c r="D654" s="1"/>
-    </row>
-    <row r="655" ht="15.75" customHeight="1">
-      <c r="B655" s="1"/>
-      <c r="C655" s="1"/>
-      <c r="D655" s="1"/>
-    </row>
-    <row r="656" ht="15.75" customHeight="1">
-      <c r="B656" s="1"/>
-      <c r="C656" s="1"/>
-      <c r="D656" s="1"/>
-    </row>
-    <row r="657" ht="15.75" customHeight="1">
-      <c r="B657" s="1"/>
-      <c r="C657" s="1"/>
-      <c r="D657" s="1"/>
-    </row>
-    <row r="658" ht="15.75" customHeight="1">
-      <c r="B658" s="1"/>
-      <c r="C658" s="1"/>
-      <c r="D658" s="1"/>
-    </row>
-    <row r="659" ht="15.75" customHeight="1">
-      <c r="B659" s="1"/>
-      <c r="C659" s="1"/>
-      <c r="D659" s="1"/>
-    </row>
-    <row r="660" ht="15.75" customHeight="1">
-      <c r="B660" s="1"/>
-      <c r="C660" s="1"/>
-      <c r="D660" s="1"/>
-    </row>
-    <row r="661" ht="15.75" customHeight="1">
-      <c r="B661" s="1"/>
-      <c r="C661" s="1"/>
-      <c r="D661" s="1"/>
-    </row>
-    <row r="662" ht="15.75" customHeight="1">
-      <c r="B662" s="1"/>
-      <c r="C662" s="1"/>
-      <c r="D662" s="1"/>
-    </row>
-    <row r="663" ht="15.75" customHeight="1">
-      <c r="B663" s="1"/>
-      <c r="C663" s="1"/>
-      <c r="D663" s="1"/>
-    </row>
-    <row r="664" ht="15.75" customHeight="1">
-      <c r="B664" s="1"/>
-      <c r="C664" s="1"/>
-      <c r="D664" s="1"/>
-    </row>
-    <row r="665" ht="15.75" customHeight="1">
-      <c r="B665" s="1"/>
-      <c r="C665" s="1"/>
-      <c r="D665" s="1"/>
-    </row>
-    <row r="666" ht="15.75" customHeight="1">
-      <c r="B666" s="1"/>
-      <c r="C666" s="1"/>
-      <c r="D666" s="1"/>
-    </row>
-    <row r="667" ht="15.75" customHeight="1">
-      <c r="B667" s="1"/>
-      <c r="C667" s="1"/>
-      <c r="D667" s="1"/>
-    </row>
-    <row r="668" ht="15.75" customHeight="1">
-      <c r="B668" s="1"/>
-      <c r="C668" s="1"/>
-      <c r="D668" s="1"/>
-    </row>
-    <row r="669" ht="15.75" customHeight="1">
-      <c r="B669" s="1"/>
-      <c r="C669" s="1"/>
-      <c r="D669" s="1"/>
-    </row>
-    <row r="670" ht="15.75" customHeight="1">
-      <c r="B670" s="1"/>
-      <c r="C670" s="1"/>
-      <c r="D670" s="1"/>
-    </row>
-    <row r="671" ht="15.75" customHeight="1">
-      <c r="B671" s="1"/>
-      <c r="C671" s="1"/>
-      <c r="D671" s="1"/>
-    </row>
-    <row r="672" ht="15.75" customHeight="1">
-      <c r="B672" s="1"/>
-      <c r="C672" s="1"/>
-      <c r="D672" s="1"/>
-    </row>
-    <row r="673" ht="15.75" customHeight="1">
-      <c r="B673" s="1"/>
-      <c r="C673" s="1"/>
-      <c r="D673" s="1"/>
-    </row>
-    <row r="674" ht="15.75" customHeight="1">
-      <c r="B674" s="1"/>
-      <c r="C674" s="1"/>
-      <c r="D674" s="1"/>
-    </row>
-    <row r="675" ht="15.75" customHeight="1">
-      <c r="B675" s="1"/>
-      <c r="C675" s="1"/>
-      <c r="D675" s="1"/>
-    </row>
-    <row r="676" ht="15.75" customHeight="1">
-      <c r="B676" s="1"/>
-      <c r="C676" s="1"/>
-      <c r="D676" s="1"/>
-    </row>
-    <row r="677" ht="15.75" customHeight="1">
-      <c r="B677" s="1"/>
-      <c r="C677" s="1"/>
-      <c r="D677" s="1"/>
-    </row>
-    <row r="678" ht="15.75" customHeight="1">
-      <c r="B678" s="1"/>
-      <c r="C678" s="1"/>
-      <c r="D678" s="1"/>
-    </row>
-    <row r="679" ht="15.75" customHeight="1">
-      <c r="B679" s="1"/>
-      <c r="C679" s="1"/>
-      <c r="D679" s="1"/>
-    </row>
-    <row r="680" ht="15.75" customHeight="1">
-      <c r="B680" s="1"/>
-      <c r="C680" s="1"/>
-      <c r="D680" s="1"/>
-    </row>
-    <row r="681" ht="15.75" customHeight="1">
-      <c r="B681" s="1"/>
-      <c r="C681" s="1"/>
-      <c r="D681" s="1"/>
-    </row>
-    <row r="682" ht="15.75" customHeight="1">
-      <c r="B682" s="1"/>
-      <c r="C682" s="1"/>
-      <c r="D682" s="1"/>
-    </row>
-    <row r="683" ht="15.75" customHeight="1">
-      <c r="B683" s="1"/>
-      <c r="C683" s="1"/>
-      <c r="D683" s="1"/>
-    </row>
-    <row r="684" ht="15.75" customHeight="1">
-      <c r="B684" s="1"/>
-      <c r="C684" s="1"/>
-      <c r="D684" s="1"/>
-    </row>
-    <row r="685" ht="15.75" customHeight="1">
-      <c r="B685" s="1"/>
-      <c r="C685" s="1"/>
-      <c r="D685" s="1"/>
-    </row>
-    <row r="686" ht="15.75" customHeight="1">
-      <c r="B686" s="1"/>
-      <c r="C686" s="1"/>
-      <c r="D686" s="1"/>
-    </row>
-    <row r="687" ht="15.75" customHeight="1">
-      <c r="B687" s="1"/>
-      <c r="C687" s="1"/>
-      <c r="D687" s="1"/>
-    </row>
-    <row r="688" ht="15.75" customHeight="1">
-      <c r="B688" s="1"/>
-      <c r="C688" s="1"/>
-      <c r="D688" s="1"/>
-    </row>
-    <row r="689" ht="15.75" customHeight="1">
-      <c r="B689" s="1"/>
-      <c r="C689" s="1"/>
-      <c r="D689" s="1"/>
-    </row>
-    <row r="690" ht="15.75" customHeight="1">
-      <c r="B690" s="1"/>
-      <c r="C690" s="1"/>
-      <c r="D690" s="1"/>
-    </row>
-    <row r="691" ht="15.75" customHeight="1">
-      <c r="B691" s="1"/>
-      <c r="C691" s="1"/>
-      <c r="D691" s="1"/>
-    </row>
-    <row r="692" ht="15.75" customHeight="1">
-      <c r="B692" s="1"/>
-      <c r="C692" s="1"/>
-      <c r="D692" s="1"/>
-    </row>
-    <row r="693" ht="15.75" customHeight="1">
-      <c r="B693" s="1"/>
-      <c r="C693" s="1"/>
-      <c r="D693" s="1"/>
-    </row>
-    <row r="694" ht="15.75" customHeight="1">
-      <c r="B694" s="1"/>
-      <c r="C694" s="1"/>
-      <c r="D694" s="1"/>
-    </row>
-    <row r="695" ht="15.75" customHeight="1">
-      <c r="B695" s="1"/>
-      <c r="C695" s="1"/>
-      <c r="D695" s="1"/>
-    </row>
-    <row r="696" ht="15.75" customHeight="1">
-      <c r="B696" s="1"/>
-      <c r="C696" s="1"/>
-      <c r="D696" s="1"/>
-    </row>
-    <row r="697" ht="15.75" customHeight="1">
-      <c r="B697" s="1"/>
-      <c r="C697" s="1"/>
-      <c r="D697" s="1"/>
-    </row>
-    <row r="698" ht="15.75" customHeight="1">
-      <c r="B698" s="1"/>
-      <c r="C698" s="1"/>
-      <c r="D698" s="1"/>
-    </row>
-    <row r="699" ht="15.75" customHeight="1">
-      <c r="B699" s="1"/>
-      <c r="C699" s="1"/>
-      <c r="D699" s="1"/>
-    </row>
-    <row r="700" ht="15.75" customHeight="1">
-      <c r="B700" s="1"/>
-      <c r="C700" s="1"/>
-      <c r="D700" s="1"/>
-    </row>
-    <row r="701" ht="15.75" customHeight="1">
-      <c r="B701" s="1"/>
-      <c r="C701" s="1"/>
-      <c r="D701" s="1"/>
-    </row>
-    <row r="702" ht="15.75" customHeight="1">
-      <c r="B702" s="1"/>
-      <c r="C702" s="1"/>
-      <c r="D702" s="1"/>
-    </row>
-    <row r="703" ht="15.75" customHeight="1">
-      <c r="B703" s="1"/>
-      <c r="C703" s="1"/>
-      <c r="D703" s="1"/>
-    </row>
-    <row r="704" ht="15.75" customHeight="1">
-      <c r="B704" s="1"/>
-      <c r="C704" s="1"/>
-      <c r="D704" s="1"/>
-    </row>
-    <row r="705" ht="15.75" customHeight="1">
-      <c r="B705" s="1"/>
-      <c r="C705" s="1"/>
-      <c r="D705" s="1"/>
-    </row>
-    <row r="706" ht="15.75" customHeight="1">
-      <c r="B706" s="1"/>
-      <c r="C706" s="1"/>
-      <c r="D706" s="1"/>
-    </row>
-    <row r="707" ht="15.75" customHeight="1">
-      <c r="B707" s="1"/>
-      <c r="C707" s="1"/>
-      <c r="D707" s="1"/>
-    </row>
-    <row r="708" ht="15.75" customHeight="1">
-      <c r="B708" s="1"/>
-      <c r="C708" s="1"/>
-      <c r="D708" s="1"/>
-    </row>
-    <row r="709" ht="15.75" customHeight="1">
-      <c r="B709" s="1"/>
-      <c r="C709" s="1"/>
-      <c r="D709" s="1"/>
-    </row>
-    <row r="710" ht="15.75" customHeight="1">
-      <c r="B710" s="1"/>
-      <c r="C710" s="1"/>
-      <c r="D710" s="1"/>
-    </row>
-    <row r="711" ht="15.75" customHeight="1">
-      <c r="B711" s="1"/>
-      <c r="C711" s="1"/>
-      <c r="D711" s="1"/>
-    </row>
-    <row r="712" ht="15.75" customHeight="1">
-      <c r="B712" s="1"/>
-      <c r="C712" s="1"/>
-      <c r="D712" s="1"/>
-    </row>
-    <row r="713" ht="15.75" customHeight="1">
-      <c r="B713" s="1"/>
-      <c r="C713" s="1"/>
-      <c r="D713" s="1"/>
-    </row>
-    <row r="714" ht="15.75" customHeight="1">
-      <c r="B714" s="1"/>
-      <c r="C714" s="1"/>
-      <c r="D714" s="1"/>
-    </row>
-    <row r="715" ht="15.75" customHeight="1">
-      <c r="B715" s="1"/>
-      <c r="C715" s="1"/>
-      <c r="D715" s="1"/>
-    </row>
-    <row r="716" ht="15.75" customHeight="1">
-      <c r="B716" s="1"/>
-      <c r="C716" s="1"/>
-      <c r="D716" s="1"/>
-    </row>
-    <row r="717" ht="15.75" customHeight="1">
-      <c r="B717" s="1"/>
-      <c r="C717" s="1"/>
-      <c r="D717" s="1"/>
-    </row>
-    <row r="718" ht="15.75" customHeight="1">
-      <c r="B718" s="1"/>
-      <c r="C718" s="1"/>
-      <c r="D718" s="1"/>
-    </row>
-    <row r="719" ht="15.75" customHeight="1">
-      <c r="B719" s="1"/>
-      <c r="C719" s="1"/>
-      <c r="D719" s="1"/>
-    </row>
-    <row r="720" ht="15.75" customHeight="1">
-      <c r="B720" s="1"/>
-      <c r="C720" s="1"/>
-      <c r="D720" s="1"/>
-    </row>
-    <row r="721" ht="15.75" customHeight="1">
-      <c r="B721" s="1"/>
-      <c r="C721" s="1"/>
-      <c r="D721" s="1"/>
-    </row>
-    <row r="722" ht="15.75" customHeight="1">
-      <c r="B722" s="1"/>
-      <c r="C722" s="1"/>
-      <c r="D722" s="1"/>
-    </row>
-    <row r="723" ht="15.75" customHeight="1">
-      <c r="B723" s="1"/>
-      <c r="C723" s="1"/>
-      <c r="D723" s="1"/>
-    </row>
-    <row r="724" ht="15.75" customHeight="1">
-      <c r="B724" s="1"/>
-      <c r="C724" s="1"/>
-      <c r="D724" s="1"/>
-    </row>
-    <row r="725" ht="15.75" customHeight="1">
-      <c r="B725" s="1"/>
-      <c r="C725" s="1"/>
-      <c r="D725" s="1"/>
-    </row>
-    <row r="726" ht="15.75" customHeight="1">
-      <c r="B726" s="1"/>
-      <c r="C726" s="1"/>
-      <c r="D726" s="1"/>
-    </row>
-    <row r="727" ht="15.75" customHeight="1">
-      <c r="B727" s="1"/>
-      <c r="C727" s="1"/>
-      <c r="D727" s="1"/>
-    </row>
-    <row r="728" ht="15.75" customHeight="1">
-      <c r="B728" s="1"/>
-      <c r="C728" s="1"/>
-      <c r="D728" s="1"/>
-    </row>
-    <row r="729" ht="15.75" customHeight="1">
-      <c r="B729" s="1"/>
-      <c r="C729" s="1"/>
-      <c r="D729" s="1"/>
-    </row>
-    <row r="730" ht="15.75" customHeight="1">
-      <c r="B730" s="1"/>
-      <c r="C730" s="1"/>
-      <c r="D730" s="1"/>
-    </row>
-    <row r="731" ht="15.75" customHeight="1">
-      <c r="B731" s="1"/>
-      <c r="C731" s="1"/>
-      <c r="D731" s="1"/>
-    </row>
-    <row r="732" ht="15.75" customHeight="1">
-      <c r="B732" s="1"/>
-      <c r="C732" s="1"/>
-      <c r="D732" s="1"/>
-    </row>
-    <row r="733" ht="15.75" customHeight="1">
-      <c r="B733" s="1"/>
-      <c r="C733" s="1"/>
-      <c r="D733" s="1"/>
-    </row>
-    <row r="734" ht="15.75" customHeight="1">
-      <c r="B734" s="1"/>
-      <c r="C734" s="1"/>
-      <c r="D734" s="1"/>
-    </row>
-    <row r="735" ht="15.75" customHeight="1">
-      <c r="B735" s="1"/>
-      <c r="C735" s="1"/>
-      <c r="D735" s="1"/>
-    </row>
-    <row r="736" ht="15.75" customHeight="1">
-      <c r="B736" s="1"/>
-      <c r="C736" s="1"/>
-      <c r="D736" s="1"/>
-    </row>
-    <row r="737" ht="15.75" customHeight="1">
-      <c r="B737" s="1"/>
-      <c r="C737" s="1"/>
-      <c r="D737" s="1"/>
-    </row>
-    <row r="738" ht="15.75" customHeight="1">
-      <c r="B738" s="1"/>
-      <c r="C738" s="1"/>
-      <c r="D738" s="1"/>
-    </row>
-    <row r="739" ht="15.75" customHeight="1">
-      <c r="B739" s="1"/>
-      <c r="C739" s="1"/>
-      <c r="D739" s="1"/>
-    </row>
-    <row r="740" ht="15.75" customHeight="1">
-      <c r="B740" s="1"/>
-      <c r="C740" s="1"/>
-      <c r="D740" s="1"/>
-    </row>
-    <row r="741" ht="15.75" customHeight="1">
-      <c r="B741" s="1"/>
-      <c r="C741" s="1"/>
-      <c r="D741" s="1"/>
-    </row>
-    <row r="742" ht="15.75" customHeight="1">
-      <c r="B742" s="1"/>
-      <c r="C742" s="1"/>
-      <c r="D742" s="1"/>
-    </row>
-    <row r="743" ht="15.75" customHeight="1">
-      <c r="B743" s="1"/>
-      <c r="C743" s="1"/>
-      <c r="D743" s="1"/>
-    </row>
-    <row r="744" ht="15.75" customHeight="1">
-      <c r="B744" s="1"/>
-      <c r="C744" s="1"/>
-      <c r="D744" s="1"/>
-    </row>
-    <row r="745" ht="15.75" customHeight="1">
-      <c r="B745" s="1"/>
-      <c r="C745" s="1"/>
-      <c r="D745" s="1"/>
-    </row>
-    <row r="746" ht="15.75" customHeight="1">
-      <c r="B746" s="1"/>
-      <c r="C746" s="1"/>
-      <c r="D746" s="1"/>
-    </row>
-    <row r="747" ht="15.75" customHeight="1">
-      <c r="B747" s="1"/>
-      <c r="C747" s="1"/>
-      <c r="D747" s="1"/>
-    </row>
-    <row r="748" ht="15.75" customHeight="1">
-      <c r="B748" s="1"/>
-      <c r="C748" s="1"/>
-      <c r="D748" s="1"/>
-    </row>
-    <row r="749" ht="15.75" customHeight="1">
-      <c r="B749" s="1"/>
-      <c r="C749" s="1"/>
-      <c r="D749" s="1"/>
-    </row>
-    <row r="750" ht="15.75" customHeight="1">
-      <c r="B750" s="1"/>
-      <c r="C750" s="1"/>
-      <c r="D750" s="1"/>
-    </row>
-    <row r="751" ht="15.75" customHeight="1">
-      <c r="B751" s="1"/>
-      <c r="C751" s="1"/>
-      <c r="D751" s="1"/>
-    </row>
-    <row r="752" ht="15.75" customHeight="1">
-      <c r="B752" s="1"/>
-      <c r="C752" s="1"/>
-      <c r="D752" s="1"/>
-    </row>
-    <row r="753" ht="15.75" customHeight="1">
-      <c r="B753" s="1"/>
-      <c r="C753" s="1"/>
-      <c r="D753" s="1"/>
-    </row>
-    <row r="754" ht="15.75" customHeight="1">
-      <c r="B754" s="1"/>
-      <c r="C754" s="1"/>
-      <c r="D754" s="1"/>
-    </row>
-    <row r="755" ht="15.75" customHeight="1">
-      <c r="B755" s="1"/>
-      <c r="C755" s="1"/>
-      <c r="D755" s="1"/>
-    </row>
-    <row r="756" ht="15.75" customHeight="1">
-      <c r="B756" s="1"/>
-      <c r="C756" s="1"/>
-      <c r="D756" s="1"/>
-    </row>
-    <row r="757" ht="15.75" customHeight="1">
-      <c r="B757" s="1"/>
-      <c r="C757" s="1"/>
-      <c r="D757" s="1"/>
-    </row>
-    <row r="758" ht="15.75" customHeight="1">
-      <c r="B758" s="1"/>
-      <c r="C758" s="1"/>
-      <c r="D758" s="1"/>
-    </row>
-    <row r="759" ht="15.75" customHeight="1">
-      <c r="B759" s="1"/>
-      <c r="C759" s="1"/>
-      <c r="D759" s="1"/>
-    </row>
-    <row r="760" ht="15.75" customHeight="1">
-      <c r="B760" s="1"/>
-      <c r="C760" s="1"/>
-      <c r="D760" s="1"/>
-    </row>
-    <row r="761" ht="15.75" customHeight="1">
-      <c r="B761" s="1"/>
-      <c r="C761" s="1"/>
-      <c r="D761" s="1"/>
-    </row>
-    <row r="762" ht="15.75" customHeight="1">
-      <c r="B762" s="1"/>
-      <c r="C762" s="1"/>
-      <c r="D762" s="1"/>
-    </row>
-    <row r="763" ht="15.75" customHeight="1">
-      <c r="B763" s="1"/>
-      <c r="C763" s="1"/>
-      <c r="D763" s="1"/>
-    </row>
-    <row r="764" ht="15.75" customHeight="1">
-      <c r="B764" s="1"/>
-      <c r="C764" s="1"/>
-      <c r="D764" s="1"/>
-    </row>
-    <row r="765" ht="15.75" customHeight="1">
-      <c r="B765" s="1"/>
-      <c r="C765" s="1"/>
-      <c r="D765" s="1"/>
-    </row>
-    <row r="766" ht="15.75" customHeight="1">
-      <c r="B766" s="1"/>
-      <c r="C766" s="1"/>
-      <c r="D766" s="1"/>
-    </row>
-    <row r="767" ht="15.75" customHeight="1">
-      <c r="B767" s="1"/>
-      <c r="C767" s="1"/>
-      <c r="D767" s="1"/>
-    </row>
-    <row r="768" ht="15.75" customHeight="1">
-      <c r="B768" s="1"/>
-      <c r="C768" s="1"/>
-      <c r="D768" s="1"/>
-    </row>
-    <row r="769" ht="15.75" customHeight="1">
-      <c r="B769" s="1"/>
-      <c r="C769" s="1"/>
-      <c r="D769" s="1"/>
-    </row>
-    <row r="770" ht="15.75" customHeight="1">
-      <c r="B770" s="1"/>
-      <c r="C770" s="1"/>
-      <c r="D770" s="1"/>
-    </row>
-    <row r="771" ht="15.75" customHeight="1">
-      <c r="B771" s="1"/>
-      <c r="C771" s="1"/>
-      <c r="D771" s="1"/>
-    </row>
-    <row r="772" ht="15.75" customHeight="1">
-      <c r="B772" s="1"/>
-      <c r="C772" s="1"/>
-      <c r="D772" s="1"/>
-    </row>
-    <row r="773" ht="15.75" customHeight="1">
-      <c r="B773" s="1"/>
-      <c r="C773" s="1"/>
-      <c r="D773" s="1"/>
-    </row>
-    <row r="774" ht="15.75" customHeight="1">
-      <c r="B774" s="1"/>
-      <c r="C774" s="1"/>
-      <c r="D774" s="1"/>
-    </row>
-    <row r="775" ht="15.75" customHeight="1">
-      <c r="B775" s="1"/>
-      <c r="C775" s="1"/>
-      <c r="D775" s="1"/>
-    </row>
-    <row r="776" ht="15.75" customHeight="1">
-      <c r="B776" s="1"/>
-      <c r="C776" s="1"/>
-      <c r="D776" s="1"/>
-    </row>
-    <row r="777" ht="15.75" customHeight="1">
-      <c r="B777" s="1"/>
-      <c r="C777" s="1"/>
-      <c r="D777" s="1"/>
-    </row>
-    <row r="778" ht="15.75" customHeight="1">
-      <c r="B778" s="1"/>
-      <c r="C778" s="1"/>
-      <c r="D778" s="1"/>
-    </row>
-    <row r="779" ht="15.75" customHeight="1">
-      <c r="B779" s="1"/>
-      <c r="C779" s="1"/>
-      <c r="D779" s="1"/>
-    </row>
-    <row r="780" ht="15.75" customHeight="1">
-      <c r="B780" s="1"/>
-      <c r="C780" s="1"/>
-      <c r="D780" s="1"/>
-    </row>
-    <row r="781" ht="15.75" customHeight="1">
-      <c r="B781" s="1"/>
-      <c r="C781" s="1"/>
-      <c r="D781" s="1"/>
-    </row>
-    <row r="782" ht="15.75" customHeight="1">
-      <c r="B782" s="1"/>
-      <c r="C782" s="1"/>
-      <c r="D782" s="1"/>
-    </row>
-    <row r="783" ht="15.75" customHeight="1">
-      <c r="B783" s="1"/>
-      <c r="C783" s="1"/>
-      <c r="D783" s="1"/>
-    </row>
-    <row r="784" ht="15.75" customHeight="1">
-      <c r="B784" s="1"/>
-      <c r="C784" s="1"/>
-      <c r="D784" s="1"/>
-    </row>
-    <row r="785" ht="15.75" customHeight="1">
-      <c r="B785" s="1"/>
-      <c r="C785" s="1"/>
-      <c r="D785" s="1"/>
-    </row>
-    <row r="786" ht="15.75" customHeight="1">
-      <c r="B786" s="1"/>
-      <c r="C786" s="1"/>
-      <c r="D786" s="1"/>
-    </row>
-    <row r="787" ht="15.75" customHeight="1">
-      <c r="B787" s="1"/>
-      <c r="C787" s="1"/>
-      <c r="D787" s="1"/>
-    </row>
-    <row r="788" ht="15.75" customHeight="1">
-      <c r="B788" s="1"/>
-      <c r="C788" s="1"/>
-      <c r="D788" s="1"/>
-    </row>
-    <row r="789" ht="15.75" customHeight="1">
-      <c r="B789" s="1"/>
-      <c r="C789" s="1"/>
-      <c r="D789" s="1"/>
-    </row>
-    <row r="790" ht="15.75" customHeight="1">
-      <c r="B790" s="1"/>
-      <c r="C790" s="1"/>
-      <c r="D790" s="1"/>
-    </row>
-    <row r="791" ht="15.75" customHeight="1">
-      <c r="B791" s="1"/>
-      <c r="C791" s="1"/>
-      <c r="D791" s="1"/>
-    </row>
-    <row r="792" ht="15.75" customHeight="1">
-      <c r="B792" s="1"/>
-      <c r="C792" s="1"/>
-      <c r="D792" s="1"/>
-    </row>
-    <row r="793" ht="15.75" customHeight="1">
-      <c r="B793" s="1"/>
-      <c r="C793" s="1"/>
-      <c r="D793" s="1"/>
-    </row>
-    <row r="794" ht="15.75" customHeight="1">
-      <c r="B794" s="1"/>
-      <c r="C794" s="1"/>
-      <c r="D794" s="1"/>
-    </row>
-    <row r="795" ht="15.75" customHeight="1">
-      <c r="B795" s="1"/>
-      <c r="C795" s="1"/>
-      <c r="D795" s="1"/>
-    </row>
-    <row r="796" ht="15.75" customHeight="1">
-      <c r="B796" s="1"/>
-      <c r="C796" s="1"/>
-      <c r="D796" s="1"/>
-    </row>
-    <row r="797" ht="15.75" customHeight="1">
-      <c r="B797" s="1"/>
-      <c r="C797" s="1"/>
-      <c r="D797" s="1"/>
-    </row>
-    <row r="798" ht="15.75" customHeight="1">
-      <c r="B798" s="1"/>
-      <c r="C798" s="1"/>
-      <c r="D798" s="1"/>
-    </row>
-    <row r="799" ht="15.75" customHeight="1">
-      <c r="B799" s="1"/>
-      <c r="C799" s="1"/>
-      <c r="D799" s="1"/>
-    </row>
-    <row r="800" ht="15.75" customHeight="1">
-      <c r="B800" s="1"/>
-      <c r="C800" s="1"/>
-      <c r="D800" s="1"/>
-    </row>
-    <row r="801" ht="15.75" customHeight="1">
-      <c r="B801" s="1"/>
-      <c r="C801" s="1"/>
-      <c r="D801" s="1"/>
-    </row>
-    <row r="802" ht="15.75" customHeight="1">
-      <c r="B802" s="1"/>
-      <c r="C802" s="1"/>
-      <c r="D802" s="1"/>
-    </row>
-    <row r="803" ht="15.75" customHeight="1">
-      <c r="B803" s="1"/>
-      <c r="C803" s="1"/>
-      <c r="D803" s="1"/>
-    </row>
-    <row r="804" ht="15.75" customHeight="1">
-      <c r="B804" s="1"/>
-      <c r="C804" s="1"/>
-      <c r="D804" s="1"/>
-    </row>
-    <row r="805" ht="15.75" customHeight="1">
-      <c r="B805" s="1"/>
-      <c r="C805" s="1"/>
-      <c r="D805" s="1"/>
-    </row>
-    <row r="806" ht="15.75" customHeight="1">
-      <c r="B806" s="1"/>
-      <c r="C806" s="1"/>
-      <c r="D806" s="1"/>
-    </row>
-    <row r="807" ht="15.75" customHeight="1">
-      <c r="B807" s="1"/>
-      <c r="C807" s="1"/>
-      <c r="D807" s="1"/>
-    </row>
-    <row r="808" ht="15.75" customHeight="1">
-      <c r="B808" s="1"/>
-      <c r="C808" s="1"/>
-      <c r="D808" s="1"/>
-    </row>
-    <row r="809" ht="15.75" customHeight="1">
-      <c r="B809" s="1"/>
-      <c r="C809" s="1"/>
-      <c r="D809" s="1"/>
-    </row>
-    <row r="810" ht="15.75" customHeight="1">
-      <c r="B810" s="1"/>
-      <c r="C810" s="1"/>
-      <c r="D810" s="1"/>
-    </row>
-    <row r="811" ht="15.75" customHeight="1">
-      <c r="B811" s="1"/>
-      <c r="C811" s="1"/>
-      <c r="D811" s="1"/>
-    </row>
-    <row r="812" ht="15.75" customHeight="1">
-      <c r="B812" s="1"/>
-      <c r="C812" s="1"/>
-      <c r="D812" s="1"/>
-    </row>
-    <row r="813" ht="15.75" customHeight="1">
-      <c r="B813" s="1"/>
-      <c r="C813" s="1"/>
-      <c r="D813" s="1"/>
-    </row>
-    <row r="814" ht="15.75" customHeight="1">
-      <c r="B814" s="1"/>
-      <c r="C814" s="1"/>
-      <c r="D814" s="1"/>
-    </row>
-    <row r="815" ht="15.75" customHeight="1">
-      <c r="B815" s="1"/>
-      <c r="C815" s="1"/>
-      <c r="D815" s="1"/>
-    </row>
-    <row r="816" ht="15.75" customHeight="1">
-      <c r="B816" s="1"/>
-      <c r="C816" s="1"/>
-      <c r="D816" s="1"/>
-    </row>
-    <row r="817" ht="15.75" customHeight="1">
-      <c r="B817" s="1"/>
-      <c r="C817" s="1"/>
-      <c r="D817" s="1"/>
-    </row>
-    <row r="818" ht="15.75" customHeight="1">
-      <c r="B818" s="1"/>
-      <c r="C818" s="1"/>
-      <c r="D818" s="1"/>
-    </row>
-    <row r="819" ht="15.75" customHeight="1">
-      <c r="B819" s="1"/>
-      <c r="C819" s="1"/>
-      <c r="D819" s="1"/>
-    </row>
-    <row r="820" ht="15.75" customHeight="1">
-      <c r="B820" s="1"/>
-      <c r="C820" s="1"/>
-      <c r="D820" s="1"/>
-    </row>
-    <row r="821" ht="15.75" customHeight="1">
-      <c r="B821" s="1"/>
-      <c r="C821" s="1"/>
-      <c r="D821" s="1"/>
-    </row>
-    <row r="822" ht="15.75" customHeight="1">
-      <c r="B822" s="1"/>
-      <c r="C822" s="1"/>
-      <c r="D822" s="1"/>
-    </row>
-    <row r="823" ht="15.75" customHeight="1">
-      <c r="B823" s="1"/>
-      <c r="C823" s="1"/>
-      <c r="D823" s="1"/>
-    </row>
-    <row r="824" ht="15.75" customHeight="1">
-      <c r="B824" s="1"/>
-      <c r="C824" s="1"/>
-      <c r="D824" s="1"/>
-    </row>
-    <row r="825" ht="15.75" customHeight="1">
-      <c r="B825" s="1"/>
-      <c r="C825" s="1"/>
-      <c r="D825" s="1"/>
-    </row>
-    <row r="826" ht="15.75" customHeight="1">
-      <c r="B826" s="1"/>
-      <c r="C826" s="1"/>
-      <c r="D826" s="1"/>
-    </row>
-    <row r="827" ht="15.75" customHeight="1">
-      <c r="B827" s="1"/>
-      <c r="C827" s="1"/>
-      <c r="D827" s="1"/>
-    </row>
-    <row r="828" ht="15.75" customHeight="1">
-      <c r="B828" s="1"/>
-      <c r="C828" s="1"/>
-      <c r="D828" s="1"/>
-    </row>
-    <row r="829" ht="15.75" customHeight="1">
-      <c r="B829" s="1"/>
-      <c r="C829" s="1"/>
-      <c r="D829" s="1"/>
-    </row>
-    <row r="830" ht="15.75" customHeight="1">
-      <c r="B830" s="1"/>
-      <c r="C830" s="1"/>
-      <c r="D830" s="1"/>
-    </row>
-    <row r="831" ht="15.75" customHeight="1">
-      <c r="B831" s="1"/>
-      <c r="C831" s="1"/>
-      <c r="D831" s="1"/>
-    </row>
-    <row r="832" ht="15.75" customHeight="1">
-      <c r="B832" s="1"/>
-      <c r="C832" s="1"/>
-      <c r="D832" s="1"/>
-    </row>
-    <row r="833" ht="15.75" customHeight="1">
-      <c r="B833" s="1"/>
-      <c r="C833" s="1"/>
-      <c r="D833" s="1"/>
-    </row>
-    <row r="834" ht="15.75" customHeight="1">
-      <c r="B834" s="1"/>
-      <c r="C834" s="1"/>
-      <c r="D834" s="1"/>
-    </row>
-    <row r="835" ht="15.75" customHeight="1">
-      <c r="B835" s="1"/>
-      <c r="C835" s="1"/>
-      <c r="D835" s="1"/>
-    </row>
-    <row r="836" ht="15.75" customHeight="1">
-      <c r="B836" s="1"/>
-      <c r="C836" s="1"/>
-      <c r="D836" s="1"/>
-    </row>
-    <row r="837" ht="15.75" customHeight="1">
-      <c r="B837" s="1"/>
-      <c r="C837" s="1"/>
-      <c r="D837" s="1"/>
-    </row>
-    <row r="838" ht="15.75" customHeight="1">
-      <c r="B838" s="1"/>
-      <c r="C838" s="1"/>
-      <c r="D838" s="1"/>
-    </row>
-    <row r="839" ht="15.75" customHeight="1">
-      <c r="B839" s="1"/>
-      <c r="C839" s="1"/>
-      <c r="D839" s="1"/>
-    </row>
-    <row r="840" ht="15.75" customHeight="1">
-      <c r="B840" s="1"/>
-      <c r="C840" s="1"/>
-      <c r="D840" s="1"/>
-    </row>
-    <row r="841" ht="15.75" customHeight="1">
-      <c r="B841" s="1"/>
-      <c r="C841" s="1"/>
-      <c r="D841" s="1"/>
-    </row>
-    <row r="842" ht="15.75" customHeight="1">
-      <c r="B842" s="1"/>
-      <c r="C842" s="1"/>
-      <c r="D842" s="1"/>
-    </row>
-    <row r="843" ht="15.75" customHeight="1">
-      <c r="B843" s="1"/>
-      <c r="C843" s="1"/>
-      <c r="D843" s="1"/>
-    </row>
-    <row r="844" ht="15.75" customHeight="1">
-      <c r="B844" s="1"/>
-      <c r="C844" s="1"/>
-      <c r="D844" s="1"/>
-    </row>
-    <row r="845" ht="15.75" customHeight="1">
-      <c r="B845" s="1"/>
-      <c r="C845" s="1"/>
-      <c r="D845" s="1"/>
-    </row>
-    <row r="846" ht="15.75" customHeight="1">
-      <c r="B846" s="1"/>
-      <c r="C846" s="1"/>
-      <c r="D846" s="1"/>
-    </row>
-    <row r="847" ht="15.75" customHeight="1">
-      <c r="B847" s="1"/>
-      <c r="C847" s="1"/>
-      <c r="D847" s="1"/>
-    </row>
-    <row r="848" ht="15.75" customHeight="1">
-      <c r="B848" s="1"/>
-      <c r="C848" s="1"/>
-      <c r="D848" s="1"/>
-    </row>
-    <row r="849" ht="15.75" customHeight="1">
-      <c r="B849" s="1"/>
-      <c r="C849" s="1"/>
-      <c r="D849" s="1"/>
-    </row>
-    <row r="850" ht="15.75" customHeight="1">
-      <c r="B850" s="1"/>
-      <c r="C850" s="1"/>
-      <c r="D850" s="1"/>
-    </row>
-    <row r="851" ht="15.75" customHeight="1">
-      <c r="B851" s="1"/>
-      <c r="C851" s="1"/>
-      <c r="D851" s="1"/>
-    </row>
-    <row r="852" ht="15.75" customHeight="1">
-      <c r="B852" s="1"/>
-      <c r="C852" s="1"/>
-      <c r="D852" s="1"/>
-    </row>
-    <row r="853" ht="15.75" customHeight="1">
-      <c r="B853" s="1"/>
-      <c r="C853" s="1"/>
-      <c r="D853" s="1"/>
-    </row>
-    <row r="854" ht="15.75" customHeight="1">
-      <c r="B854" s="1"/>
-      <c r="C854" s="1"/>
-      <c r="D854" s="1"/>
-    </row>
-    <row r="855" ht="15.75" customHeight="1">
-      <c r="B855" s="1"/>
-      <c r="C855" s="1"/>
-      <c r="D855" s="1"/>
-    </row>
-    <row r="856" ht="15.75" customHeight="1">
-      <c r="B856" s="1"/>
-      <c r="C856" s="1"/>
-      <c r="D856" s="1"/>
-    </row>
-    <row r="857" ht="15.75" customHeight="1">
-      <c r="B857" s="1"/>
-      <c r="C857" s="1"/>
-      <c r="D857" s="1"/>
-    </row>
-    <row r="858" ht="15.75" customHeight="1">
-      <c r="B858" s="1"/>
-      <c r="C858" s="1"/>
-      <c r="D858" s="1"/>
-    </row>
-    <row r="859" ht="15.75" customHeight="1">
-      <c r="B859" s="1"/>
-      <c r="C859" s="1"/>
-      <c r="D859" s="1"/>
-    </row>
-    <row r="860" ht="15.75" customHeight="1">
-      <c r="B860" s="1"/>
-      <c r="C860" s="1"/>
-      <c r="D860" s="1"/>
-    </row>
-    <row r="861" ht="15.75" customHeight="1">
-      <c r="B861" s="1"/>
-      <c r="C861" s="1"/>
-      <c r="D861" s="1"/>
-    </row>
-    <row r="862" ht="15.75" customHeight="1">
-      <c r="B862" s="1"/>
-      <c r="C862" s="1"/>
-      <c r="D862" s="1"/>
-    </row>
-    <row r="863" ht="15.75" customHeight="1">
-      <c r="B863" s="1"/>
-      <c r="C863" s="1"/>
-      <c r="D863" s="1"/>
-    </row>
-    <row r="864" ht="15.75" customHeight="1">
-      <c r="B864" s="1"/>
-      <c r="C864" s="1"/>
-      <c r="D864" s="1"/>
-    </row>
-    <row r="865" ht="15.75" customHeight="1">
-      <c r="B865" s="1"/>
-      <c r="C865" s="1"/>
-      <c r="D865" s="1"/>
-    </row>
-    <row r="866" ht="15.75" customHeight="1">
-      <c r="B866" s="1"/>
-      <c r="C866" s="1"/>
-      <c r="D866" s="1"/>
-    </row>
-    <row r="867" ht="15.75" customHeight="1">
-      <c r="B867" s="1"/>
-      <c r="C867" s="1"/>
-      <c r="D867" s="1"/>
-    </row>
-    <row r="868" ht="15.75" customHeight="1">
-      <c r="B868" s="1"/>
-      <c r="C868" s="1"/>
-      <c r="D868" s="1"/>
-    </row>
-    <row r="869" ht="15.75" customHeight="1">
-      <c r="B869" s="1"/>
-      <c r="C869" s="1"/>
-      <c r="D869" s="1"/>
-    </row>
-    <row r="870" ht="15.75" customHeight="1">
-      <c r="B870" s="1"/>
-      <c r="C870" s="1"/>
-      <c r="D870" s="1"/>
-    </row>
-    <row r="871" ht="15.75" customHeight="1">
-      <c r="B871" s="1"/>
-      <c r="C871" s="1"/>
-      <c r="D871" s="1"/>
-    </row>
-    <row r="872" ht="15.75" customHeight="1">
-      <c r="B872" s="1"/>
-      <c r="C872" s="1"/>
-      <c r="D872" s="1"/>
-    </row>
-    <row r="873" ht="15.75" customHeight="1">
-      <c r="B873" s="1"/>
-      <c r="C873" s="1"/>
-      <c r="D873" s="1"/>
-    </row>
-    <row r="874" ht="15.75" customHeight="1">
-      <c r="B874" s="1"/>
-      <c r="C874" s="1"/>
-      <c r="D874" s="1"/>
-    </row>
-    <row r="875" ht="15.75" customHeight="1">
-      <c r="B875" s="1"/>
-      <c r="C875" s="1"/>
-      <c r="D875" s="1"/>
-    </row>
-    <row r="876" ht="15.75" customHeight="1">
-      <c r="B876" s="1"/>
-      <c r="C876" s="1"/>
-      <c r="D876" s="1"/>
-    </row>
-    <row r="877" ht="15.75" customHeight="1">
-      <c r="B877" s="1"/>
-      <c r="C877" s="1"/>
-      <c r="D877" s="1"/>
-    </row>
-    <row r="878" ht="15.75" customHeight="1">
-      <c r="B878" s="1"/>
-      <c r="C878" s="1"/>
-      <c r="D878" s="1"/>
-    </row>
-    <row r="879" ht="15.75" customHeight="1">
-      <c r="B879" s="1"/>
-      <c r="C879" s="1"/>
-      <c r="D879" s="1"/>
-    </row>
-    <row r="880" ht="15.75" customHeight="1">
-      <c r="B880" s="1"/>
-      <c r="C880" s="1"/>
-      <c r="D880" s="1"/>
-    </row>
-    <row r="881" ht="15.75" customHeight="1">
-      <c r="B881" s="1"/>
-      <c r="C881" s="1"/>
-      <c r="D881" s="1"/>
-    </row>
-    <row r="882" ht="15.75" customHeight="1">
-      <c r="B882" s="1"/>
-      <c r="C882" s="1"/>
-      <c r="D882" s="1"/>
-    </row>
-    <row r="883" ht="15.75" customHeight="1">
-      <c r="B883" s="1"/>
-      <c r="C883" s="1"/>
-      <c r="D883" s="1"/>
-    </row>
-    <row r="884" ht="15.75" customHeight="1">
-      <c r="B884" s="1"/>
-      <c r="C884" s="1"/>
-      <c r="D884" s="1"/>
-    </row>
-    <row r="885" ht="15.75" customHeight="1">
-      <c r="B885" s="1"/>
-      <c r="C885" s="1"/>
-      <c r="D885" s="1"/>
-    </row>
-    <row r="886" ht="15.75" customHeight="1">
-      <c r="B886" s="1"/>
-      <c r="C886" s="1"/>
-      <c r="D886" s="1"/>
-    </row>
-    <row r="887" ht="15.75" customHeight="1">
-      <c r="B887" s="1"/>
-      <c r="C887" s="1"/>
-      <c r="D887" s="1"/>
-    </row>
-    <row r="888" ht="15.75" customHeight="1">
-      <c r="B888" s="1"/>
-      <c r="C888" s="1"/>
-      <c r="D888" s="1"/>
-    </row>
-    <row r="889" ht="15.75" customHeight="1">
-      <c r="B889" s="1"/>
-      <c r="C889" s="1"/>
-      <c r="D889" s="1"/>
-    </row>
-    <row r="890" ht="15.75" customHeight="1">
-      <c r="B890" s="1"/>
-      <c r="C890" s="1"/>
-      <c r="D890" s="1"/>
-    </row>
-    <row r="891" ht="15.75" customHeight="1">
-      <c r="B891" s="1"/>
-      <c r="C891" s="1"/>
-      <c r="D891" s="1"/>
-    </row>
-    <row r="892" ht="15.75" customHeight="1">
-      <c r="B892" s="1"/>
-      <c r="C892" s="1"/>
-      <c r="D892" s="1"/>
-    </row>
-    <row r="893" ht="15.75" customHeight="1">
-      <c r="B893" s="1"/>
-      <c r="C893" s="1"/>
-      <c r="D893" s="1"/>
-    </row>
-    <row r="894" ht="15.75" customHeight="1">
-      <c r="B894" s="1"/>
-      <c r="C894" s="1"/>
-      <c r="D894" s="1"/>
-    </row>
-    <row r="895" ht="15.75" customHeight="1">
-      <c r="B895" s="1"/>
-      <c r="C895" s="1"/>
-      <c r="D895" s="1"/>
-    </row>
-    <row r="896" ht="15.75" customHeight="1">
-      <c r="B896" s="1"/>
-      <c r="C896" s="1"/>
-      <c r="D896" s="1"/>
-    </row>
-    <row r="897" ht="15.75" customHeight="1">
-      <c r="B897" s="1"/>
-      <c r="C897" s="1"/>
-      <c r="D897" s="1"/>
-    </row>
-    <row r="898" ht="15.75" customHeight="1">
-      <c r="B898" s="1"/>
-      <c r="C898" s="1"/>
-      <c r="D898" s="1"/>
-    </row>
-    <row r="899" ht="15.75" customHeight="1">
-      <c r="B899" s="1"/>
-      <c r="C899" s="1"/>
-      <c r="D899" s="1"/>
-    </row>
-    <row r="900" ht="15.75" customHeight="1">
-      <c r="B900" s="1"/>
-      <c r="C900" s="1"/>
-      <c r="D900" s="1"/>
-    </row>
-    <row r="901" ht="15.75" customHeight="1">
-      <c r="B901" s="1"/>
-      <c r="C901" s="1"/>
-      <c r="D901" s="1"/>
-    </row>
-    <row r="902" ht="15.75" customHeight="1">
-      <c r="B902" s="1"/>
-      <c r="C902" s="1"/>
-      <c r="D902" s="1"/>
-    </row>
-    <row r="903" ht="15.75" customHeight="1">
-      <c r="B903" s="1"/>
-      <c r="C903" s="1"/>
-      <c r="D903" s="1"/>
-    </row>
-    <row r="904" ht="15.75" customHeight="1">
-      <c r="B904" s="1"/>
-      <c r="C904" s="1"/>
-      <c r="D904" s="1"/>
-    </row>
-    <row r="905" ht="15.75" customHeight="1">
-      <c r="B905" s="1"/>
-      <c r="C905" s="1"/>
-      <c r="D905" s="1"/>
-    </row>
-    <row r="906" ht="15.75" customHeight="1">
-      <c r="B906" s="1"/>
-      <c r="C906" s="1"/>
-      <c r="D906" s="1"/>
-    </row>
-    <row r="907" ht="15.75" customHeight="1">
-      <c r="B907" s="1"/>
-      <c r="C907" s="1"/>
-      <c r="D907" s="1"/>
-    </row>
-    <row r="908" ht="15.75" customHeight="1">
-      <c r="B908" s="1"/>
-      <c r="C908" s="1"/>
-      <c r="D908" s="1"/>
-    </row>
-    <row r="909" ht="15.75" customHeight="1">
-      <c r="B909" s="1"/>
-      <c r="C909" s="1"/>
-      <c r="D909" s="1"/>
-    </row>
-    <row r="910" ht="15.75" customHeight="1">
-      <c r="B910" s="1"/>
-      <c r="C910" s="1"/>
-      <c r="D910" s="1"/>
-    </row>
-    <row r="911" ht="15.75" customHeight="1">
-      <c r="B911" s="1"/>
-      <c r="C911" s="1"/>
-      <c r="D911" s="1"/>
-    </row>
-    <row r="912" ht="15.75" customHeight="1">
-      <c r="B912" s="1"/>
-      <c r="C912" s="1"/>
-      <c r="D912" s="1"/>
-    </row>
-    <row r="913" ht="15.75" customHeight="1">
-      <c r="B913" s="1"/>
-      <c r="C913" s="1"/>
-      <c r="D913" s="1"/>
-    </row>
-    <row r="914" ht="15.75" customHeight="1">
-      <c r="B914" s="1"/>
-      <c r="C914" s="1"/>
-      <c r="D914" s="1"/>
-    </row>
-    <row r="915" ht="15.75" customHeight="1">
-      <c r="B915" s="1"/>
-      <c r="C915" s="1"/>
-      <c r="D915" s="1"/>
-    </row>
-    <row r="916" ht="15.75" customHeight="1">
-      <c r="B916" s="1"/>
-      <c r="C916" s="1"/>
-      <c r="D916" s="1"/>
-    </row>
-    <row r="917" ht="15.75" customHeight="1">
-      <c r="B917" s="1"/>
-      <c r="C917" s="1"/>
-      <c r="D917" s="1"/>
-    </row>
-    <row r="918" ht="15.75" customHeight="1">
-      <c r="B918" s="1"/>
-      <c r="C918" s="1"/>
-      <c r="D918" s="1"/>
-    </row>
-    <row r="919" ht="15.75" customHeight="1">
-      <c r="B919" s="1"/>
-      <c r="C919" s="1"/>
-      <c r="D919" s="1"/>
-    </row>
-    <row r="920" ht="15.75" customHeight="1">
-      <c r="B920" s="1"/>
-      <c r="C920" s="1"/>
-      <c r="D920" s="1"/>
-    </row>
-    <row r="921" ht="15.75" customHeight="1">
-      <c r="B921" s="1"/>
-      <c r="C921" s="1"/>
-      <c r="D921" s="1"/>
-    </row>
-    <row r="922" ht="15.75" customHeight="1">
-      <c r="B922" s="1"/>
-      <c r="C922" s="1"/>
-      <c r="D922" s="1"/>
-    </row>
-    <row r="923" ht="15.75" customHeight="1">
-      <c r="B923" s="1"/>
-      <c r="C923" s="1"/>
-      <c r="D923" s="1"/>
-    </row>
-    <row r="924" ht="15.75" customHeight="1">
-      <c r="B924" s="1"/>
-      <c r="C924" s="1"/>
-      <c r="D924" s="1"/>
-    </row>
-    <row r="925" ht="15.75" customHeight="1">
-      <c r="B925" s="1"/>
-      <c r="C925" s="1"/>
-      <c r="D925" s="1"/>
-    </row>
-    <row r="926" ht="15.75" customHeight="1">
-      <c r="B926" s="1"/>
-      <c r="C926" s="1"/>
-      <c r="D926" s="1"/>
-    </row>
-    <row r="927" ht="15.75" customHeight="1">
-      <c r="B927" s="1"/>
-      <c r="C927" s="1"/>
-      <c r="D927" s="1"/>
-    </row>
-    <row r="928" ht="15.75" customHeight="1">
-      <c r="B928" s="1"/>
-      <c r="C928" s="1"/>
-      <c r="D928" s="1"/>
-    </row>
-    <row r="929" ht="15.75" customHeight="1">
-      <c r="B929" s="1"/>
-      <c r="C929" s="1"/>
-      <c r="D929" s="1"/>
-    </row>
-    <row r="930" ht="15.75" customHeight="1">
-      <c r="B930" s="1"/>
-      <c r="C930" s="1"/>
-      <c r="D930" s="1"/>
-    </row>
-    <row r="931" ht="15.75" customHeight="1">
-      <c r="B931" s="1"/>
-      <c r="C931" s="1"/>
-      <c r="D931" s="1"/>
-    </row>
-    <row r="932" ht="15.75" customHeight="1">
-      <c r="B932" s="1"/>
-      <c r="C932" s="1"/>
-      <c r="D932" s="1"/>
-    </row>
-    <row r="933" ht="15.75" customHeight="1">
-      <c r="B933" s="1"/>
-      <c r="C933" s="1"/>
-      <c r="D933" s="1"/>
-    </row>
-    <row r="934" ht="15.75" customHeight="1">
-      <c r="B934" s="1"/>
-      <c r="C934" s="1"/>
-      <c r="D934" s="1"/>
-    </row>
-    <row r="935" ht="15.75" customHeight="1">
-      <c r="B935" s="1"/>
-      <c r="C935" s="1"/>
-      <c r="D935" s="1"/>
-    </row>
-    <row r="936" ht="15.75" customHeight="1">
-      <c r="B936" s="1"/>
-      <c r="C936" s="1"/>
-      <c r="D936" s="1"/>
-    </row>
-    <row r="937" ht="15.75" customHeight="1">
-      <c r="B937" s="1"/>
-      <c r="C937" s="1"/>
-      <c r="D937" s="1"/>
-    </row>
-    <row r="938" ht="15.75" customHeight="1">
-      <c r="B938" s="1"/>
-      <c r="C938" s="1"/>
-      <c r="D938" s="1"/>
-    </row>
-    <row r="939" ht="15.75" customHeight="1">
-      <c r="B939" s="1"/>
-      <c r="C939" s="1"/>
-      <c r="D939" s="1"/>
-    </row>
-    <row r="940" ht="15.75" customHeight="1">
-      <c r="B940" s="1"/>
-      <c r="C940" s="1"/>
-      <c r="D940" s="1"/>
-    </row>
-    <row r="941" ht="15.75" customHeight="1">
-      <c r="B941" s="1"/>
-      <c r="C941" s="1"/>
-      <c r="D941" s="1"/>
-    </row>
-    <row r="942" ht="15.75" customHeight="1">
-      <c r="B942" s="1"/>
-      <c r="C942" s="1"/>
-      <c r="D942" s="1"/>
-    </row>
-    <row r="943" ht="15.75" customHeight="1">
-      <c r="B943" s="1"/>
-      <c r="C943" s="1"/>
-      <c r="D943" s="1"/>
-    </row>
-    <row r="944" ht="15.75" customHeight="1">
-      <c r="B944" s="1"/>
-      <c r="C944" s="1"/>
-      <c r="D944" s="1"/>
-    </row>
-    <row r="945" ht="15.75" customHeight="1">
-      <c r="B945" s="1"/>
-      <c r="C945" s="1"/>
-      <c r="D945" s="1"/>
-    </row>
-    <row r="946" ht="15.75" customHeight="1">
-      <c r="B946" s="1"/>
-      <c r="C946" s="1"/>
-      <c r="D946" s="1"/>
-    </row>
-    <row r="947" ht="15.75" customHeight="1">
-      <c r="B947" s="1"/>
-      <c r="C947" s="1"/>
-      <c r="D947" s="1"/>
-    </row>
-    <row r="948" ht="15.75" customHeight="1">
-      <c r="B948" s="1"/>
-      <c r="C948" s="1"/>
-      <c r="D948" s="1"/>
-    </row>
-    <row r="949" ht="15.75" customHeight="1">
-      <c r="B949" s="1"/>
-      <c r="C949" s="1"/>
-      <c r="D949" s="1"/>
-    </row>
-    <row r="950" ht="15.75" customHeight="1">
-      <c r="B950" s="1"/>
-      <c r="C950" s="1"/>
-      <c r="D950" s="1"/>
-    </row>
-    <row r="951" ht="15.75" customHeight="1">
-      <c r="B951" s="1"/>
-      <c r="C951" s="1"/>
-      <c r="D951" s="1"/>
-    </row>
-    <row r="952" ht="15.75" customHeight="1">
-      <c r="B952" s="1"/>
-      <c r="C952" s="1"/>
-      <c r="D952" s="1"/>
-    </row>
-    <row r="953" ht="15.75" customHeight="1">
-      <c r="B953" s="1"/>
-      <c r="C953" s="1"/>
-      <c r="D953" s="1"/>
-    </row>
-    <row r="954" ht="15.75" customHeight="1">
-      <c r="B954" s="1"/>
-      <c r="C954" s="1"/>
-      <c r="D954" s="1"/>
-    </row>
-    <row r="955" ht="15.75" customHeight="1">
-      <c r="B955" s="1"/>
-      <c r="C955" s="1"/>
-      <c r="D955" s="1"/>
-    </row>
-    <row r="956" ht="15.75" customHeight="1">
-      <c r="B956" s="1"/>
-      <c r="C956" s="1"/>
-      <c r="D956" s="1"/>
-    </row>
-    <row r="957" ht="15.75" customHeight="1">
-      <c r="B957" s="1"/>
-      <c r="C957" s="1"/>
-      <c r="D957" s="1"/>
-    </row>
-    <row r="958" ht="15.75" customHeight="1">
-      <c r="B958" s="1"/>
-      <c r="C958" s="1"/>
-      <c r="D958" s="1"/>
-    </row>
-    <row r="959" ht="15.75" customHeight="1">
-      <c r="B959" s="1"/>
-      <c r="C959" s="1"/>
-      <c r="D959" s="1"/>
-    </row>
-    <row r="960" ht="15.75" customHeight="1">
-      <c r="B960" s="1"/>
-      <c r="C960" s="1"/>
-      <c r="D960" s="1"/>
-    </row>
-    <row r="961" ht="15.75" customHeight="1">
-      <c r="B961" s="1"/>
-      <c r="C961" s="1"/>
-      <c r="D961" s="1"/>
-    </row>
-    <row r="962" ht="15.75" customHeight="1">
-      <c r="B962" s="1"/>
-      <c r="C962" s="1"/>
-      <c r="D962" s="1"/>
-    </row>
-    <row r="963" ht="15.75" customHeight="1">
-      <c r="B963" s="1"/>
-      <c r="C963" s="1"/>
-      <c r="D963" s="1"/>
-    </row>
-    <row r="964" ht="15.75" customHeight="1">
-      <c r="B964" s="1"/>
-      <c r="C964" s="1"/>
-      <c r="D964" s="1"/>
-    </row>
-    <row r="965" ht="15.75" customHeight="1">
-      <c r="B965" s="1"/>
-      <c r="C965" s="1"/>
-      <c r="D965" s="1"/>
-    </row>
-    <row r="966" ht="15.75" customHeight="1">
-      <c r="B966" s="1"/>
-      <c r="C966" s="1"/>
-      <c r="D966" s="1"/>
-    </row>
-    <row r="967" ht="15.75" customHeight="1">
-      <c r="B967" s="1"/>
-      <c r="C967" s="1"/>
-      <c r="D967" s="1"/>
-    </row>
-    <row r="968" ht="15.75" customHeight="1">
-      <c r="B968" s="1"/>
-      <c r="C968" s="1"/>
-      <c r="D968" s="1"/>
-    </row>
-    <row r="969" ht="15.75" customHeight="1">
-      <c r="B969" s="1"/>
-      <c r="C969" s="1"/>
-      <c r="D969" s="1"/>
-    </row>
-    <row r="970" ht="15.75" customHeight="1">
-      <c r="B970" s="1"/>
-      <c r="C970" s="1"/>
-      <c r="D970" s="1"/>
-    </row>
-    <row r="971" ht="15.75" customHeight="1">
-      <c r="B971" s="1"/>
-      <c r="C971" s="1"/>
-      <c r="D971" s="1"/>
-    </row>
-    <row r="972" ht="15.75" customHeight="1">
-      <c r="B972" s="1"/>
-      <c r="C972" s="1"/>
-      <c r="D972" s="1"/>
-    </row>
-    <row r="973" ht="15.75" customHeight="1">
-      <c r="B973" s="1"/>
-      <c r="C973" s="1"/>
-      <c r="D973" s="1"/>
-    </row>
-    <row r="974" ht="15.75" customHeight="1">
-      <c r="B974" s="1"/>
-      <c r="C974" s="1"/>
-      <c r="D974" s="1"/>
-    </row>
-    <row r="975" ht="15.75" customHeight="1">
-      <c r="B975" s="1"/>
-      <c r="C975" s="1"/>
-      <c r="D975" s="1"/>
-    </row>
-    <row r="976" ht="15.75" customHeight="1">
-      <c r="B976" s="1"/>
-      <c r="C976" s="1"/>
-      <c r="D976" s="1"/>
-    </row>
-    <row r="977" ht="15.75" customHeight="1">
-      <c r="B977" s="1"/>
-      <c r="C977" s="1"/>
-      <c r="D977" s="1"/>
-    </row>
-    <row r="978" ht="15.75" customHeight="1">
-      <c r="B978" s="1"/>
-      <c r="C978" s="1"/>
-      <c r="D978" s="1"/>
-    </row>
-    <row r="979" ht="15.75" customHeight="1">
-      <c r="B979" s="1"/>
-      <c r="C979" s="1"/>
-      <c r="D979" s="1"/>
-    </row>
-    <row r="980" ht="15.75" customHeight="1">
-      <c r="B980" s="1"/>
-      <c r="C980" s="1"/>
-      <c r="D980" s="1"/>
-    </row>
-    <row r="981" ht="15.75" customHeight="1">
-      <c r="B981" s="1"/>
-      <c r="C981" s="1"/>
-      <c r="D981" s="1"/>
-    </row>
-    <row r="982" ht="15.75" customHeight="1">
-      <c r="B982" s="1"/>
-      <c r="C982" s="1"/>
-      <c r="D982" s="1"/>
-    </row>
-    <row r="983" ht="15.75" customHeight="1">
-      <c r="B983" s="1"/>
-      <c r="C983" s="1"/>
-      <c r="D983" s="1"/>
-    </row>
-    <row r="984" ht="15.75" customHeight="1">
-      <c r="B984" s="1"/>
-      <c r="C984" s="1"/>
-      <c r="D984" s="1"/>
-    </row>
-    <row r="985" ht="15.75" customHeight="1">
-      <c r="B985" s="1"/>
-      <c r="C985" s="1"/>
-      <c r="D985" s="1"/>
-    </row>
-    <row r="986" ht="15.75" customHeight="1">
-      <c r="B986" s="1"/>
-      <c r="C986" s="1"/>
-      <c r="D986" s="1"/>
-    </row>
-    <row r="987" ht="15.75" customHeight="1">
-      <c r="B987" s="1"/>
-      <c r="C987" s="1"/>
-      <c r="D987" s="1"/>
-    </row>
-    <row r="988" ht="15.75" customHeight="1">
-      <c r="B988" s="1"/>
-      <c r="C988" s="1"/>
-      <c r="D988" s="1"/>
-    </row>
-    <row r="989" ht="15.75" customHeight="1">
-      <c r="B989" s="1"/>
-      <c r="C989" s="1"/>
-      <c r="D989" s="1"/>
-    </row>
-    <row r="990" ht="15.75" customHeight="1">
-      <c r="B990" s="1"/>
-      <c r="C990" s="1"/>
-      <c r="D990" s="1"/>
-    </row>
-    <row r="991" ht="15.75" customHeight="1">
-      <c r="B991" s="1"/>
-      <c r="C991" s="1"/>
-      <c r="D991" s="1"/>
-    </row>
-    <row r="992" ht="15.75" customHeight="1">
-      <c r="B992" s="1"/>
-      <c r="C992" s="1"/>
-      <c r="D992" s="1"/>
-    </row>
-    <row r="993" ht="15.75" customHeight="1">
-      <c r="B993" s="1"/>
-      <c r="C993" s="1"/>
-      <c r="D993" s="1"/>
-    </row>
-    <row r="994" ht="15.75" customHeight="1">
-      <c r="B994" s="1"/>
-      <c r="C994" s="1"/>
-      <c r="D994" s="1"/>
-    </row>
-    <row r="995" ht="15.75" customHeight="1">
-      <c r="B995" s="1"/>
-      <c r="C995" s="1"/>
-      <c r="D995" s="1"/>
-    </row>
-    <row r="996" ht="15.75" customHeight="1">
-      <c r="B996" s="1"/>
-      <c r="C996" s="1"/>
-      <c r="D996" s="1"/>
-    </row>
-    <row r="997" ht="15.75" customHeight="1">
-      <c r="B997" s="1"/>
-      <c r="C997" s="1"/>
-      <c r="D997" s="1"/>
-    </row>
-    <row r="998" ht="15.75" customHeight="1">
-      <c r="B998" s="1"/>
-      <c r="C998" s="1"/>
-      <c r="D998" s="1"/>
-    </row>
-    <row r="999" ht="15.75" customHeight="1">
-      <c r="B999" s="1"/>
-      <c r="C999" s="1"/>
-      <c r="D999" s="1"/>
-    </row>
-    <row r="1000" ht="15.75" customHeight="1">
-      <c r="B1000" s="1"/>
-      <c r="C1000" s="1"/>
-      <c r="D1000" s="1"/>
-    </row>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -7211,7 +4679,7 @@
       <c r="C4" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>171</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -7220,474 +4688,474 @@
       <c r="F4" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="6"/>
-      <c r="Z4" s="6"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="5"/>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="D5" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="D6" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7" t="s">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" s="8" t="s">
+      <c r="D7" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F8" s="8" t="s">
+      <c r="D8" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" s="8" t="s">
+      <c r="D9" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F10" s="8" t="s">
+      <c r="D10" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="8" t="s">
+      <c r="D11" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" s="8" t="s">
+      <c r="D12" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F13" s="8" t="s">
+      <c r="D13" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F14" s="8" t="s">
+      <c r="D14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7" t="s">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F15" s="8" t="s">
+      <c r="D15" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" s="8" t="s">
+      <c r="D16" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F17" s="8" t="s">
+      <c r="D17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" s="8" t="s">
+      <c r="D18" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F19" s="8" t="s">
+      <c r="D19" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7" t="s">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="8" t="s">
+      <c r="D20" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7" t="s">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="8" t="s">
+      <c r="D21" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F22" s="8" t="s">
+      <c r="D22" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7" t="s">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D23" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F23" s="8" t="s">
+      <c r="D23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="D24" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F24" s="8" t="s">
+      <c r="D24" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="D25" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F25" s="8" t="s">
+      <c r="D25" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F25" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7" t="s">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="D26" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F26" s="8" t="s">
+      <c r="D26" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F26" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7" t="s">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D27" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F27" s="8" t="s">
+      <c r="D27" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7" t="s">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F28" s="8" t="s">
+      <c r="D28" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7" t="s">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F29" s="8" t="s">
+      <c r="D29" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>108</v>
       </c>
     </row>
@@ -7708,7 +5176,7 @@
       <c r="C33" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="4" t="s">
         <v>214</v>
       </c>
       <c r="E33" s="4" t="s">
@@ -7719,50 +5187,52 @@
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7" t="s">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F34" s="8" t="s">
+      <c r="C34" s="6"/>
+      <c r="D34" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7" t="s">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F35" s="8" t="s">
+      <c r="C35" s="6"/>
+      <c r="D35" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7" t="s">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F36" s="9"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
@@ -8747,7 +6217,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="8.71"/>
+    <col customWidth="1" min="1" max="6" width="8.71"/>
   </cols>
   <sheetData>
     <row r="2">

</xml_diff>